<commit_message>
new branch for testing development
</commit_message>
<xml_diff>
--- a/results/chatbot-results.xlsx
+++ b/results/chatbot-results.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G20"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -433,7 +433,7 @@
         <v>All</v>
       </c>
       <c r="D2" t="str">
-        <v>What are the IB approaches to learning?</v>
+        <v>when do the new enhancement guides come out</v>
       </c>
       <c r="E2" t="str">
         <v/>
@@ -442,7 +442,7 @@
         <v>PASS</v>
       </c>
       <c r="G2" t="str">
-        <v>2026-09-17T04:43:58.281Z</v>
+        <v>2026-09-17T13:30:27.092Z</v>
       </c>
     </row>
     <row r="3" xml:space="preserve">
@@ -456,37 +456,427 @@
         <v>All</v>
       </c>
       <c r="D3" t="str">
-        <v>What is the IB learner profile?</v>
+        <v>how does a stduent make use of a bilingual dictionary?</v>
       </c>
       <c r="E3" t="str" xml:space="preserve">
-        <v xml:space="preserve">Overview
-The IB learner profile is a statement of the qualities the International Baccalaureate aims to develop in students — a broad set of intellectual, personal, emotional and social attributes that put the IB mission into practice and support the development of internationally minded, active and caring citizens. The profile is intended to inspire and guide students, teachers and whole-school communities in what they are trying to achieve with and for learners. 1 2 3
-The ten attributes
-Inquirers
-Knowledgeable
-Thinkers
-Communicators
-Principled
-Open‑minded
-Caring
-Risk‑takers
-Balanced
-Reflective
-These 10 attributes are described as dispositions, understandings and skills that are developed progressively across IB programmes and used as a common language for reflection and growth. 3 1
-Development and implementation
-The attributes are intended to be developed over time in many contexts (classroom inquiry, service, language learning and community engagement) and documented in curriculum planning and assessment practices. Schools have some permitted implementation options (for example, replacing “risk‑taker” with “courageous” or, within the descriptor of “balanced,” adding the word “spiritual”); schools may also add additional attributes aligned with the IB mission if they follow the IB’s guidance on naming and justification. The learner profile is routinely integrated into unit planners, programme guidance and whole‑school approaches to support student progression. 1 4
-1The learner_the-learner-en_a698410d-e95a-452f-bc70-ecc544da2ae4.xml_92What is an IB education?_what-is-an-ib-education-en_148279a4-dd5d-4552-bd1c-187c8442d91c.xml_23Mathematics: Frequently asked questions from the webinar “How to help your students thrive during the MYP mathematics eAssessment”_m_5_mathm_faq_2403_1_e.pdf_24What is an IB education? support material_what-is-an-ib-education-support-material-en_8e64a303-5f54-4de8-861e-4e6afb31c104.xml_9</v>
+        <v xml:space="preserve">A student can make use of a bilingual dictionary to support their language learning by facilitating understanding and communication between their first language and the new language they are acquiring. It helps in clarifying vocabulary meanings, checking translations, and supporting comprehension in both languages. Using a bilingual dictionary aligns with the additive approach to bilingual education, where the student's first language is valued and developed alongside the new language, reinforcing cognitive and linguistic growth. This tool can aid students in navigating bilingual programmes effectively and enhances their overall language proficiency by supporting connections between languages 12.
+1The PYP and bilingual education_the-pyp-and-bilingual-education-en_85b2c145-2728-4a5d-b163-af143dde6134.xml_102The PYP and bilingual education_the-pyp-and-bilingual-education-en_85b2c145-2728-4a5d-b163-af143dde6134.xml_2</v>
       </c>
       <c r="F3" t="str">
         <v>PASS</v>
       </c>
       <c r="G3" t="str">
-        <v>2026-09-17T04:44:19.119Z</v>
+        <v>2026-09-17T13:30:38.999Z</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="str">
+        <v>All</v>
+      </c>
+      <c r="C4" t="str">
+        <v>All</v>
+      </c>
+      <c r="D4" t="str">
+        <v>how much are the fees for the ibdp courses</v>
+      </c>
+      <c r="E4" t="str">
+        <v>I'm sorry, I'm unable to process this request.</v>
+      </c>
+      <c r="F4" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G4" t="str">
+        <v>2026-09-17T13:30:53.739Z</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="str">
+        <v>All</v>
+      </c>
+      <c r="C5" t="str">
+        <v>All</v>
+      </c>
+      <c r="D5" t="str">
+        <v>When is it going to be?</v>
+      </c>
+      <c r="E5" t="str">
+        <v>I'm sorry, I'm unable to process this request.</v>
+      </c>
+      <c r="F5" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G5" t="str">
+        <v>2026-09-17T13:31:08.105Z</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="str">
+        <v>All</v>
+      </c>
+      <c r="C6" t="str">
+        <v>All</v>
+      </c>
+      <c r="D6" t="str">
+        <v>where can i find information regarding the types of assessment for MYP 5 Sciences criterion D</v>
+      </c>
+      <c r="E6" t="str">
+        <v>I'm sorry, I'm unable to process this request.</v>
+      </c>
+      <c r="F6" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G6" t="str">
+        <v>2026-09-17T13:31:19.611Z</v>
+      </c>
+    </row>
+    <row r="7" xml:space="preserve">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="str">
+        <v>All</v>
+      </c>
+      <c r="C7" t="str">
+        <v>All</v>
+      </c>
+      <c r="D7" t="str">
+        <v>necesito compararla con una original en español?</v>
+      </c>
+      <c r="E7" t="str" xml:space="preserve">
+        <v xml:space="preserve">Sí, se recomienda utilizar fuentes originales en la lengua objeto de estudio, en este caso el español, para evitar errores gramaticales y lingüísticos que pueden surgir de malas traducciones. Además, se aconseja no usar traductores electrónicos, ya que a menudo producen resultados incomprensibles. Esto ayuda a garantizar una mejor comprensión y precisión en el análisis y la comparación de textos 1.
+1Spanish B extended essay report, May 2012_d_2_abspa_eer_1205_1_s.pdf_5</v>
+      </c>
+      <c r="F7" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G7" t="str">
+        <v>2026-09-17T13:31:28.101Z</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="str">
+        <v>All</v>
+      </c>
+      <c r="C8" t="str">
+        <v>All</v>
+      </c>
+      <c r="D8" t="str">
+        <v>no necesito compararla con una original en español?</v>
+      </c>
+      <c r="E8" t="str">
+        <v>I'm sorry, I'm unable to process this request.</v>
+      </c>
+      <c r="F8" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G8" t="str">
+        <v>2026-09-17T13:31:40.125Z</v>
+      </c>
+    </row>
+    <row r="9" xml:space="preserve">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="str">
+        <v>All</v>
+      </c>
+      <c r="C9" t="str">
+        <v>All</v>
+      </c>
+      <c r="D9" t="str">
+        <v>No--I get the flexibility. It's one of IB's strengths. I don't think giving teachers flexibility is not the reason that the coherent philosophy and pedagogy is spread out across multiple documents, with some essential bits found in single subject guides like Psychology and Sports Exercise and Health Science</v>
+      </c>
+      <c r="E9" t="str" xml:space="preserve">
+        <v xml:space="preserve">You're correct that the IB's coherent philosophy and pedagogy are indeed distributed across multiple documents, including general programme materials as well as subject-specific guides such as those for Psychology and Sports, Exercise and Health Science. This multi-document approach ensures detailed and specialized guidance tailored to each subject while maintaining alignment with the overarching IB mission and educational principles. Flexibility for teachers is a strength of the IB, but it operates within a well-structured framework that spans these various resources to support a consistent and comprehensive educational experience 123.
+1Flexibility in the programme of inquiry_flexibility-in-the-programme-of-inquiry-en_47e60c4c-8bb3-4c31-b579-d5e96d2c003f.xml_12Philosophy teacher support material_philosophy-teacher-support-material-en_28af1d45-30b1-42ce-9173-2b932a15f7aa.xml_13Sports, exercise and health science guide (First assessment 2018)_d_4_sport_gui_1601_5_e.pdf_6</v>
+      </c>
+      <c r="F9" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G9" t="str">
+        <v>2026-09-17T13:31:55.341Z</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="str">
+        <v>All</v>
+      </c>
+      <c r="C10" t="str">
+        <v>All</v>
+      </c>
+      <c r="D10" t="str">
+        <v>que distancia tienen que haber entre alumnos para los digitales</v>
+      </c>
+      <c r="E10" t="str">
+        <v>I'm sorry, I'm unable to process this request.</v>
+      </c>
+      <c r="F10" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G10" t="str">
+        <v>2026-09-17T13:32:09.739Z</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="str">
+        <v>All</v>
+      </c>
+      <c r="C11" t="str">
+        <v>All</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Pueden usar un serie de televisión para el oral de DP inglés A lengua y literatura</v>
+      </c>
+      <c r="E11" t="str">
+        <v>I'm sorry, I'm unable to process this request.</v>
+      </c>
+      <c r="F11" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G11" t="str">
+        <v>2026-09-17T13:32:24.637Z</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="str">
+        <v>All</v>
+      </c>
+      <c r="C12" t="str">
+        <v>All</v>
+      </c>
+      <c r="D12" t="str">
+        <v>what is the assessment criteria for the art inquiries project</v>
+      </c>
+      <c r="E12" t="str">
+        <v>I'm sorry, I'm unable to process this request.</v>
+      </c>
+      <c r="F12" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G12" t="str">
+        <v>2026-09-17T13:32:36.448Z</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="str">
+        <v>All</v>
+      </c>
+      <c r="C13" t="str">
+        <v>All</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Ce sont les anciens objectifs...  Il y a 4 nouveaux objectifs. Quels sont-ils?</v>
+      </c>
+      <c r="E13" t="str">
+        <v/>
+      </c>
+      <c r="F13" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G13" t="str">
+        <v>2026-09-17T13:33:23.185Z</v>
+      </c>
+    </row>
+    <row r="14" xml:space="preserve">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="str">
+        <v>All</v>
+      </c>
+      <c r="C14" t="str">
+        <v>All</v>
+      </c>
+      <c r="D14" t="str">
+        <v>And what about first exam May 2029?</v>
+      </c>
+      <c r="E14" t="str" xml:space="preserve">
+        <v xml:space="preserve">The exact start date for the May 2029 IB examination session is not provided in the retrieved documents. However, based on the pattern from previous years, the IB examinations typically begin in late April and run through mid to late May, with no exams scheduled on 1 May. For example, the 2027 examinations start on Friday, 23 April 2027, and end on Wednesday, 19 May 2027, and the 2028 examinations start on Tuesday, 25 April 2028, and end on Friday, 19 May 2028 12. It is likely that the 2029 schedule will follow a similar timeline, but the official schedule will be confirmed closer to the date, usually a couple of years in advance.
+1May 2026 examination schedule - final version_d_0_dpyyy_sup_2404_3_26_e.pdf_102May 2027 examination schedule - final version_d_0_dpyyy_sup_2502_2_27_e.pdf_10</v>
+      </c>
+      <c r="F14" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G14" t="str">
+        <v>2026-09-17T13:33:34.970Z</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="str">
+        <v>All</v>
+      </c>
+      <c r="C15" t="str">
+        <v>All</v>
+      </c>
+      <c r="D15" t="str">
+        <v>how many criteria will be there in the myp from 2027</v>
+      </c>
+      <c r="E15" t="str">
+        <v>I'm sorry, I'm unable to process this request.</v>
+      </c>
+      <c r="F15" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G15" t="str">
+        <v>2026-09-17T13:33:51.578Z</v>
+      </c>
+    </row>
+    <row r="16" xml:space="preserve">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="str">
+        <v>All</v>
+      </c>
+      <c r="C16" t="str">
+        <v>All</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Pendant les sessions d'examens IBDP, j'ai entendu dire qu'il pouvait y avoir des pauses durant les épreuves, notamment pour certains élèves avec certaines difficultés. Si c'est vraiment le cas, peux-tu m'expliquer de manière aussi détaillée que possible comment cela peut se passer et sous quelles conditions ?</v>
+      </c>
+      <c r="E16" t="str" xml:space="preserve">
+        <v xml:space="preserve">Oui, pendant les sessions d'examens du Programme du Diplôme de l'IB (IBDP), certains élèves peuvent bénéficier de pauses (appelées "rest breaks") pendant les épreuves, notamment ceux qui rencontrent des difficultés physiques, émotionnelles ou cognitives.
+Voici comment cela peut se passer et sous quelles conditions :
+Nature des pauses : Ces pauses permettent à l'élève de se détendre, s'étirer, bouger, se rafraîchir ou pratiquer quelques minutes de pleine conscience ou méditation. Elles sont planifiées de façon à aider l'élève à déstresser, se recharger et revenir à la tâche dans de meilleures conditions.
+Organisation : Le timing et la durée des pauses sont adaptés aux besoins spécifiques de l'élève, en accord avec ce qui lui sera le plus utile pour mieux gérer le stress ou l'inconfort durant l'examen.
+Conditions d'autorisation : Ces pauses sont généralement mises en place par l'école sans nécessiter une autorisation préalable de l'IB, notamment dans des cas tels que troubles émotionnels, blessures nécessitant des changements de posture réguliers, anxiété ou autres difficultés similaires.
+Exemples concrets :
+Un élève souffrant d'une blessure au dos peut bénéficier de pauses pour changer de position toutes les 30 minutes.
+Un élève émotionnellement perturbé par des circonstances personnelles difficiles peut avoir des pauses pour sortir quelques minutes de la salle et se calmer.
+Mise en place : C’est le coordinateur de programme ou l'école qui organise ces pauses en accord avec l'élève et dans le respect des règles de conduite des examens de l'IB.
+Pas besoin d'autorisation IB : Pour ces pauses, l'approbation formelle de l'IB n'est pas requise, ce qui facilite leur mise en place rapide et adaptée.
+Pour plus de détails, ces arrangements font partie des mesures d'accommodement mises en place pour soutenir les élèves en situation d'adversité ou avec des besoins spécifiques pendant les examens 123.
+1Adverse circumstances policy_adverse-circumstances-policy-en_a16ae1f9-cbf9-442d-aeff-fc116f6d32ac.xml_22Access and inclusion planning during the COVID-19 pandemic: Access arrangements for mental health challenges_g_0_senxx_csn_2010_1c_e.pdf_43Adverse circumstances policy_adverse-circumstances-policy-en_a16ae1f9-cbf9-442d-aeff-fc116f6d32ac.xml_8</v>
+      </c>
+      <c r="F16" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G16" t="str">
+        <v>2026-09-17T13:34:10.667Z</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="str">
+        <v>All</v>
+      </c>
+      <c r="C17" t="str">
+        <v>All</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Formulario d4</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Le formulaire D4 n'est pas contenu dans les documents récupérés. Les documents fournis concernent principalement le formulaire D2, utilisé pour signaler des circonstances défavorables affectant un ou plusieurs élèves pendant les sessions d'examens IB, ainsi que les mesures compensatoires associées. Pour obtenir le formulaire D4, il est recommandé de consulter le Centre de ressources pédagogiques de l'IB ou de contacter directement le coordinateur IB de votre établissement.</v>
+      </c>
+      <c r="F17" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G17" t="str">
+        <v>2026-09-17T13:34:25.785Z</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="str">
+        <v>All</v>
+      </c>
+      <c r="C18" t="str">
+        <v>All</v>
+      </c>
+      <c r="D18" t="str">
+        <v>If they don't do it, will the IB not award them the Diploma?</v>
+      </c>
+      <c r="E18" t="str">
+        <v>I'm sorry, I'm unable to process this request.</v>
+      </c>
+      <c r="F18" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G18" t="str">
+        <v>2026-09-17T13:34:41.553Z</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="str">
+        <v>All</v>
+      </c>
+      <c r="C19" t="str">
+        <v>All</v>
+      </c>
+      <c r="D19" t="str">
+        <v>what percentage is the BM SL IA worth?</v>
+      </c>
+      <c r="E19" t="str">
+        <v>I'm sorry, I'm unable to process this request.</v>
+      </c>
+      <c r="F19" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G19" t="str">
+        <v>2026-09-17T13:34:50.059Z</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="str">
+        <v>All</v>
+      </c>
+      <c r="C20" t="str">
+        <v>All</v>
+      </c>
+      <c r="D20" t="str">
+        <v>What percentage of an DP Economics student's final grade is determined by their Internal Assessment?</v>
+      </c>
+      <c r="E20" t="str">
+        <v>locator.count: Target page, context or browser has been closed</v>
+      </c>
+      <c r="F20" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="G20" t="str">
+        <v>2026-09-17T13:34:55.784Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G20"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Increases time 1 hr to 24 hr
</commit_message>
<xml_diff>
--- a/results/chatbot-results.xlsx
+++ b/results/chatbot-results.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G61"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -422,7 +422,7 @@
         <v>timestamp</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" xml:space="preserve">
       <c r="A2">
         <v>1</v>
       </c>
@@ -433,16 +433,17 @@
         <v>All</v>
       </c>
       <c r="D2" t="str">
-        <v>What are the IB approaches to learning?</v>
-      </c>
-      <c r="E2" t="str">
-        <v/>
+        <v>What is the MYP? *</v>
+      </c>
+      <c r="E2" t="str" xml:space="preserve">
+        <v xml:space="preserve">The Middle Years Programme (MYP) is a comprehensive curriculum framework developed by the International Baccalaureate (IB) for students aged 11 to 16. It provides academic challenge and supports the development of life skills during a critical period of young people's growth, helping them build personal strengths, embrace challenges, and develop a strong sense of personal identity. The MYP emphasizes holistic learning, intercultural awareness, communication, and prepares students for further successful study. It is inclusive, designed to benefit all students, and organized around eight subject groups with a concept-driven and inquiry-based curriculum. The programme also includes important projects like the community project and personal project that develop students' skills in service and reflection, preparing them for future education and life experiences 123.
+1MYP: From principles into practice (Updated 2022 for use with the latest Programme standards and practices)_m_0_mypxx_guu_1405_10_e.pdf_62MYP: From principles into practice 2014 (For candidate schools following the 2014 Programme standards and practices authorization process)_m_0_mypxx_guu_2209_1_e.pdf_83Community project guide_myp-community-project-guide-en_1ab030ac-869b-4052-b2bd-f1bfe6aa2240.xml_2</v>
       </c>
       <c r="F2" t="str">
         <v>PASS</v>
       </c>
       <c r="G2" t="str">
-        <v>2026-09-17T04:43:58.281Z</v>
+        <v>2026-09-29T05:02:57.547Z</v>
       </c>
     </row>
     <row r="3" xml:space="preserve">
@@ -456,37 +457,1491 @@
         <v>All</v>
       </c>
       <c r="D3" t="str">
-        <v>What is the IB learner profile?</v>
+        <v>i need the descriptors ST</v>
       </c>
       <c r="E3" t="str" xml:space="preserve">
-        <v xml:space="preserve">Overview
-The IB learner profile is a statement of the qualities the International Baccalaureate aims to develop in students — a broad set of intellectual, personal, emotional and social attributes that put the IB mission into practice and support the development of internationally minded, active and caring citizens. The profile is intended to inspire and guide students, teachers and whole-school communities in what they are trying to achieve with and for learners. 1 2 3
-The ten attributes
-Inquirers
-Knowledgeable
-Thinkers
-Communicators
-Principled
-Open‑minded
-Caring
-Risk‑takers
-Balanced
-Reflective
-These 10 attributes are described as dispositions, understandings and skills that are developed progressively across IB programmes and used as a common language for reflection and growth. 3 1
-Development and implementation
-The attributes are intended to be developed over time in many contexts (classroom inquiry, service, language learning and community engagement) and documented in curriculum planning and assessment practices. Schools have some permitted implementation options (for example, replacing “risk‑taker” with “courageous” or, within the descriptor of “balanced,” adding the word “spiritual”); schools may also add additional attributes aligned with the IB mission if they follow the IB’s guidance on naming and justification. The learner profile is routinely integrated into unit planners, programme guidance and whole‑school approaches to support student progression. 1 4
-1The learner_the-learner-en_a698410d-e95a-452f-bc70-ecc544da2ae4.xml_92What is an IB education?_what-is-an-ib-education-en_148279a4-dd5d-4552-bd1c-187c8442d91c.xml_23Mathematics: Frequently asked questions from the webinar “How to help your students thrive during the MYP mathematics eAssessment”_m_5_mathm_faq_2403_1_e.pdf_24What is an IB education? support material_what-is-an-ib-education-support-material-en_8e64a303-5f54-4de8-861e-4e6afb31c104.xml_9</v>
+        <v xml:space="preserve">Subject-specific grade descriptors in the MYP serve as important references in the assessment process. They describe student performance at each grade level for each MYP subject group, aligning with criterion-related assessment philosophy. Teachers use these descriptors to predict student outcomes in eAssessment, ensuring alignment between teacher expectations and IB assessment results. The grade award team uses these descriptors to set grade boundaries, comparing student performance against descriptors at key grade transitions (e.g., grades 2 to 3, 3 to 4, and 6 to 7). This process helps standardize assessment across subjects and sessions by referencing real student work 1.
+1Interdisciplinary teaching and learning in the MYP (for use from September 2021/January 2022)_interdisciplinary-teaching-and-learning-in-the-myp-guide-en_1700f2b5-ce51-4dae-b272-c75303fca437.xml_24</v>
       </c>
       <c r="F3" t="str">
         <v>PASS</v>
       </c>
       <c r="G3" t="str">
-        <v>2026-09-17T04:44:19.119Z</v>
+        <v>2026-09-29T05:03:09.315Z</v>
+      </c>
+    </row>
+    <row r="4" xml:space="preserve">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="str">
+        <v>All</v>
+      </c>
+      <c r="C4" t="str">
+        <v>All</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Is there anything specific for PYP? AF</v>
+      </c>
+      <c r="E4" t="str" xml:space="preserve">
+        <v xml:space="preserve">Yes, the Primary Years Programme (PYP) is specifically designed for students aged 3 to 12 and focuses on the development of the whole child as an inquirer both inside and outside the classroom. It is a curriculum framework guided by six transdisciplinary themes of global significance, explored through six subject areas and approaches to learning with a strong emphasis on inquiry. The PYP supports early learning through a constructivist and social constructivist approach, encouraging active exploration and play to foster cognitive and social-emotional development. It also values early learning as a crucial stage in brain development and lifelong learning foundation. The PYP is flexible to accommodate local curriculum demands and emphasizes international-mindedness, action, and inquiry-based learning tailored to young learners' developmental needs 123.
+1PYP principles for learning and teaching (video transcript, June 2016)_p_0_pypxx_crr_1606_1_e.pdf_12The early years in the PYP_the-early-years-in-the-pyp-en_9ea4bfa4-cb65-4dae-833c-57f40d6d93b7.xml_13IB and the ELA Common Core State Standards—Relationship studies: Resources to inform curriculum alignment_g_0_iboxx_amo_1308_1e_e.pdf_4</v>
+      </c>
+      <c r="F4" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G4" t="str">
+        <v>2026-09-29T05:03:20.557Z</v>
+      </c>
+    </row>
+    <row r="5" xml:space="preserve">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="str">
+        <v>All</v>
+      </c>
+      <c r="C5" t="str">
+        <v>All</v>
+      </c>
+      <c r="D5" t="str">
+        <v>I want documents that support conceptual understanding ST</v>
+      </c>
+      <c r="E5" t="str" xml:space="preserve">
+        <v xml:space="preserve">Conceptual understanding in IB programmes, including the MYP and PYP, is a central educational goal focusing on transforming personal understanding and collaborative meaning-making rather than rote memorization. Concepts are defined as "big ideas" that are enduring and transcend specific subjects or times, enabling students to explore significant issues and ideas. They promote deeper understanding, interdisciplinary connections, and critical and creative thinking skills. In the MYP, conceptual understanding involves key and related concepts that provide both breadth and depth, helping students co-construct meaning and develop transferability of knowledge and responsibility for their learning. Teaching through concepts encourages a broad, inclusive approach to education across national and cultural boundaries, supporting interdisciplinary learning and engagement with complex ideas 1.
+1MYP: From principles into practice 2014 (For candidate schools following the 2014 Programme standards and practices authorization process)_m_0_mypxx_guu_2209_1_e.pdf_16</v>
+      </c>
+      <c r="F5" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G5" t="str">
+        <v>2026-09-29T05:03:31.777Z</v>
+      </c>
+    </row>
+    <row r="6" xml:space="preserve">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="str">
+        <v>All</v>
+      </c>
+      <c r="C6" t="str">
+        <v>All</v>
+      </c>
+      <c r="D6" t="str">
+        <v>scope and sequence \ST</v>
+      </c>
+      <c r="E6" t="str" xml:space="preserve">
+        <v xml:space="preserve">_x001b_[2mexpect(_x001b_[22m_x001b_[31mreceived_x001b_[39m_x001b_[2m)._x001b_[22mtoBeGreaterThan_x001b_[2m(_x001b_[22m_x001b_[32mexpected_x001b_[39m_x001b_[2m)_x001b_[22m
+Expected: &gt; _x001b_[32m4_x001b_[39m
+Received:   _x001b_[31m4_x001b_[39m
+Call Log:
+- Timeout 180000ms exceeded while waiting on the predicate</v>
+      </c>
+      <c r="F6" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="G6" t="str">
+        <v>2026-09-29T05:06:32.204Z</v>
+      </c>
+    </row>
+    <row r="7" xml:space="preserve">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="str">
+        <v>All</v>
+      </c>
+      <c r="C7" t="str">
+        <v>All</v>
+      </c>
+      <c r="D7" t="str">
+        <v>learning progressions ST</v>
+      </c>
+      <c r="E7" t="str" xml:space="preserve">
+        <v xml:space="preserve">Learning progressions in the IB context describe the development of skills, understanding, and capabilities as students increase their proficiency in a particular area. They serve as tools to help teachers identify students' current learning stages, recognize gaps, and plan the next achievable steps to advance learning. These progressions integrate cognitive and measurement sciences, linking curriculum, assessment, and instruction to provide coherence and support student growth. They emphasize starting from the learner's existing understanding, actively involving learners, developing metacognition, and recognizing the social aspects of learning. Learning progressions align with the IB’s emphasis on student agency and support a social constructivist approach, making learning visible and actionable for both educators and learners. Specifically, in the Primary Years Programme (PYP), learning progressions offer a framework for describing skills that represent an IB learner within subjects, supporting schools in designing customized scope and sequence documents that reflect their contexts. These progressions also act as bridges between curriculum, assessment, and pedagogy, enabling coherent and developmentally appropriate learning experiences across age groups 12345.
+1Learning progressions: Research report (April 2021)_p_0_pypxx_sur-ir_2104_1l_e.pdf_12Learning progressions: Research report (April 2021)_p_0_pypxx_sur-ir_2104_1l_e.pdf_53Learning progressions: Research report (April 2021)_p_0_pypxx_sur-ir_2104_1l_e.pdf_24Inquiry learning progressions: Introduction_inquiry-learning-progressions-introduction-en_63f5ac5f-ebbf-43e2-9d91-2ae3d88c6ca8.xml_15Learning progressions: Research report (April 2021)_p_0_pypxx_sur-ir_2104_1l_e.pdf_4</v>
+      </c>
+      <c r="F7" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G7" t="str">
+        <v>2026-09-29T05:06:43.516Z</v>
+      </c>
+    </row>
+    <row r="8" xml:space="preserve">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="str">
+        <v>All</v>
+      </c>
+      <c r="C8" t="str">
+        <v>All</v>
+      </c>
+      <c r="D8" t="str">
+        <v>I there any seperate document or a page in PYP which talks about approaches to teaching ST</v>
+      </c>
+      <c r="E8" t="str" xml:space="preserve">
+        <v xml:space="preserve">Yes, there is a specific focus on "approaches to teaching" within the Primary Years Programme (PYP). It is described as part of the curriculum cycle — written, taught, and assessed — and emphasizes authentic learning that is inquiry-based and conceptually driven. This is discussed in the context of PYP's review themes, highlighting how learning is most effective when connected to the real world around students rather than contrived school tasks 1. Additionally, the PYP: From principles into practice document elaborates on the organizing structure of the programme, including learning and teaching approaches that support learner agency and inquiry-based education 2.
+1Consultation paper: An invitation to PYP Heads, coordinators and educators at IB World Schools to comment on key themes for the PYP review process. (January 2014)_p_0_pypxx_crr_1402_1_e.pdf_12Transition guide for the Primary Years Programme_p_0_pypxx_mph_1806_1_e.pdf_2</v>
+      </c>
+      <c r="F8" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G8" t="str">
+        <v>2026-09-29T05:06:55.319Z</v>
+      </c>
+    </row>
+    <row r="9" xml:space="preserve">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="str">
+        <v>All</v>
+      </c>
+      <c r="C9" t="str">
+        <v>All</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Pyp exhibition AF</v>
+      </c>
+      <c r="E9" t="str" xml:space="preserve">
+        <v xml:space="preserve">The PYP exhibition is a significant culminating learning experience in the Primary Years Programme where students demonstrate their understanding through an in-depth inquiry into issues or opportunities they have chosen to explore. It involves students taking responsibility for their learning by planning, sharing, and assessing their work collaboratively with peers and mentors. The exhibition showcases student agency and community engagement, emphasizing international-mindedness and action. It may be integrated as one of the six units of inquiry in the final year or conducted as a separate inquiry project, with flexibility for schools to adapt it to their context. Students initiate, design, and collaborate throughout the exhibition process, developing knowledge, skills, and conceptual understanding. Assessment focuses on reflection and documentation rather than grading, and schools are encouraged to move from guided to student-led exhibitions over several years to support growing student independence 1234.
+1PYP: From principles into practice FAQs_p_0_pypxx_faq_2008_4_e.pdf_52The learner_the-learner-en_a698410d-e95a-452f-bc70-ecc544da2ae4.xml_163PYP: From principles into practice FAQs_p_0_pypxx_faq_2008_4_e.pdf_64The Learner in the enhanced PYP_p_0_pypxx_amo_1711_1_e.pdf_5</v>
+      </c>
+      <c r="F9" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G9" t="str">
+        <v>2026-09-29T05:07:10.546Z</v>
+      </c>
+    </row>
+    <row r="10" xml:space="preserve">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="str">
+        <v>All</v>
+      </c>
+      <c r="C10" t="str">
+        <v>All</v>
+      </c>
+      <c r="D10" t="str">
+        <v>what are the 5 ATL ? ST</v>
+      </c>
+      <c r="E10" t="str" xml:space="preserve">
+        <v xml:space="preserve">The five Approaches to Learning (ATL) skill categories identified in IB programmes are:
+Communication
+Social
+Self-management
+Research
+Thinking
+These categories encompass various skill clusters that help students learn how to learn, develop independence, collaborate, and reflect effectively 123.
+1Approaches to teaching and learning in the Diploma Programme_approaches-to-teaching-and-learning-in-the-diploma-programme-en_72487a02-2ee8-4cac-a7f2-3519bcd20703.xml_32Approaches to learning and approaches to teaching in the Middle Years Programme_approaches-to-learning-and-approaches-to-teaching-in-the-mid-en_af9646cb-da0c-4a76-bc1d-4c127a5b7744.xml_33MYP: From principles into practice (Updated 2022 for use with the latest Programme standards and practices)_m_0_mypxx_guu_1405_10_e.pdf_21</v>
+      </c>
+      <c r="F10" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G10" t="str">
+        <v>2026-09-29T05:07:22.097Z</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="str">
+        <v>All</v>
+      </c>
+      <c r="C11" t="str">
+        <v>All</v>
+      </c>
+      <c r="D11" t="str">
+        <v>stand alone subjects PYP  AF</v>
+      </c>
+      <c r="E11" t="str">
+        <v/>
+      </c>
+      <c r="F11" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G11" t="str">
+        <v>2026-09-29T05:08:04.527Z</v>
+      </c>
+    </row>
+    <row r="12" xml:space="preserve">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="str">
+        <v>All</v>
+      </c>
+      <c r="C12" t="str">
+        <v>All</v>
+      </c>
+      <c r="D12" t="str">
+        <v>How can schools ensure academic honesty and ethical use of AI tools such as ChatGPT in DP and MYP assessments?</v>
+      </c>
+      <c r="E12" t="str" xml:space="preserve">
+        <v xml:space="preserve">Schools can ensure academic honesty and the ethical use of AI tools like ChatGPT in DP and MYP assessments by implementing several key strategies:
+Develop and enforce an academic honesty policy aligned with IB expectations, tailored to the school's context and priorities, which clearly addresses the use of AI tools 1.
+Provide detailed guidance and staff development on academic writing, referencing systems, plagiarism, and the ethical use of AI tools to clarify expectations for both teachers and students 12.
+Require students to acknowledge AI-generated content by including in-text citations and bibliographic references specifying the AI tool used, the prompt given, and the date of generation, ensuring transparency and proper attribution 23.
+Engage students in discussions about academic integrity as an ethical choice, including the responsible use of emerging technologies, privacy, bias, and accountability, to foster critical thinking and ethical awareness 24.
+Use assessment design strategies such as selecting unique, specific, or localized topics that encourage original inquiry and reduce opportunities for plagiarism or reliance on ready-made AI outputs 1.
+Monitor and support students' use of AI tools, encouraging prompt history documentation to verify authenticity and improve students' skills in using AI responsibly 2.
+Ensure school policies on AI use are clear, communicated, and consistently applied, while teachers exercise professional judgment on the appropriate use of AI in learning and assessment contexts 524.
+Together, these approaches help maintain academic integrity while embracing the educational potential of AI technologies in IB programmes.
+1IB position paper: Academic honesty in the IB_g_0_ibres_sur-dr_1209_1a_e.pdf_62Reflective project teacher support material (first teaching 2025)_cp-reflective-project-tsm-2025-en_ac05169d-d5c9-4f6c-989f-c42854416389.xml_123Key points to explain the use of Artificial Intelligence (AI) tools (one page fact sheet)_g_0_malpr_sup_2305_2_e.pdf_14Academic integrity policy_academic-integrity-policy-en_d1fbfeab-1d1e-4349-96aa-a314410bc760.xml_255Personal and professional skills teacher support material (first teaching 2025)_cp-personal-and-professional-skills-tsm-2025-en_f0592814-2fb3-4c52-a9a5-fc63dd1ff082.xml_8</v>
+      </c>
+      <c r="F12" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G12" t="str">
+        <v>2026-09-29T05:08:18.817Z</v>
+      </c>
+    </row>
+    <row r="13" xml:space="preserve">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="str">
+        <v>All</v>
+      </c>
+      <c r="C13" t="str">
+        <v>All</v>
+      </c>
+      <c r="D13" t="str">
+        <v>will we still have related concepts</v>
+      </c>
+      <c r="E13" t="str" xml:space="preserve">
+        <v xml:space="preserve">Yes, related concepts continue to be an important part of the IB curriculum framework. In the Primary Years Programme (PYP), students encounter key and related concepts, and in the Middle Years Programme (MYP) and Diploma Programme (DP), students further develop these conceptual understandings. Related concepts support inquiry into significant ideas and help students make connections across subjects and contexts, contributing to a deeper and more connected learning experience 1.
+1MYP: From principles into practice (Updated 2022 for use with the latest Programme standards and practices)_m_0_mypxx_guu_1405_10_e.pdf_15</v>
+      </c>
+      <c r="F13" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G13" t="str">
+        <v>2026-09-29T05:08:30.512Z</v>
+      </c>
+    </row>
+    <row r="14" xml:space="preserve">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="str">
+        <v>All</v>
+      </c>
+      <c r="C14" t="str">
+        <v>All</v>
+      </c>
+      <c r="D14" t="str">
+        <v>How can an IB World School effectively implement and evaluate ATL skills, student agency, inquiry-based learning, inclusion, academic integrity, multilingualism, and ethical AI use across the PYP, MYP, and DP while ensuring alignment with IB standards, collaborative planning, assessment practices, and evaluation visit expectations?</v>
+      </c>
+      <c r="E14" t="str" xml:space="preserve">
+        <v xml:space="preserve">To effectively implement and evaluate Approaches to Learning (ATL) skills, student agency, inquiry-based learning, inclusion, academic integrity, multilingualism, and ethical AI use across PYP, MYP, and DP, an IB World School should adopt a comprehensive, collaborative, and reflective approach aligned with IB standards:
+Collaborative Planning and Integration: Schools should create time and structures for teachers to collaborate horizontally and vertically, ensuring ATL skills and other key elements are embedded consistently across subjects and year levels. This involves shared planning meetings, interdisciplinary units, and coordinated curriculum maps reflecting ATL progression and inquiry-based learning approaches 1.
+Community Involvement and Partnerships: Engaging counselors, librarians, parents, and coordinators as allies in supporting ATL development, study skills, academic honesty, and ethical practices is essential. Counselors can coach students on balance and stress management, while librarians support information literacy, academic honesty, and research skills. Parents can reinforce reflective practices and ethical use of technology at home 23.
+Clear Policies and Guidance: Developing and communicating detailed academic honesty policies aligned with IB expectations ensures learners understand integrity requirements, including managing plagiarism and appropriate use of AI tools. Providing students with guidelines on citations and ethical AI use fosters transparency and responsibility 4.
+Formative and Summative Assessment Practices: Implement assessment strategies that promote student agency and self-assessment, encouraging learners to reflect on their ATL skill development and inquiry processes. Use assessment for learning principles to adapt teaching responsively and provide meaningful feedback, supporting inclusive learning environments 53.
+Monitoring and Reflection: Regular self-assessment and reflection by students on their ATL skills and learning progress enhance motivation and ownership. Schools can include these reflections in reporting and use them to inform curriculum adjustments and professional development 3.
+Alignment with IB Standards and Evaluation: Documenting collaborative planning, ATL skill integration, academic honesty practices, and inclusive strategies provides evidence for IB programme standards and evaluation visits. Maintaining clear records of planning agendas, unit plans, policy documents, and examples of student work supports the evaluation process 14.
+By embedding these elements systematically and fostering a school-wide culture of ethical, inquiry-driven, and inclusive learning, IB World Schools can uphold IB principles and meet programme expectations effectively.
+1Further guidance for developing ATL in the MYP_m_0_mypxx_fcl_1409_1a_e.pdf_42Approaches to teaching and learning in the Diploma Programme_approaches-to-teaching-and-learning-in-the-diploma-programme-en_72487a02-2ee8-4cac-a7f2-3519bcd20703.xml_313Approaches to teaching and learning in the Diploma Programme_approaches-to-teaching-and-learning-in-the-diploma-programme-en_72487a02-2ee8-4cac-a7f2-3519bcd20703.xml_304IB position paper: Academic honesty in the IB_g_0_ibres_sur-dr_1209_1a_e.pdf_15Teaching and learning informed by assessment in the Diploma Programme_teaching-and-learning-informed-by-assessment-in-the-diploma--en_a8ba94f8-e0ea-4c2c-b2d7-c578850fec35.xml_1</v>
+      </c>
+      <c r="F14" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G14" t="str">
+        <v>2026-09-29T05:08:51.822Z</v>
+      </c>
+    </row>
+    <row r="15" xml:space="preserve">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="str">
+        <v>All</v>
+      </c>
+      <c r="C15" t="str">
+        <v>All</v>
+      </c>
+      <c r="D15" t="str">
+        <v>am I allowed to use the term "IB Prep" or "pre-IB" for classes in a junior program leading the DP, and we have MYP.</v>
+      </c>
+      <c r="E15" t="str" xml:space="preserve">
+        <v xml:space="preserve">The retrieved IB documentation does not provide specific guidelines regarding the use of terms like "IB Prep" or "pre-IB" for classes in a junior program leading to the Diploma Programme (DP), especially when the school already offers the Middle Years Programme (MYP). Generally, schools authorized to offer IB programmes follow IB terminology and frameworks to maintain clarity and alignment with IB standards.
+To ensure compliance and avoid confusion, it is recommended that schools consult directly with their IB regional office or IB coordinator for guidance on appropriate naming conventions for programs preparing students for the DP, particularly when the MYP is already offered as the official junior programme 12.
+1Middle Years Programme Assessment procedures 2025_myp-assessment-procedures-2025-en_5b9e6038-e524-4797-9e5e-57b70799783e.xml_72Middle Years Programme Assessment procedures 2026_myp-assessment-procedures-2026-en_ec81f7c7-2942-4e7c-ac96-a18447c2ca3e.xml_7</v>
+      </c>
+      <c r="F15" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G15" t="str">
+        <v>2026-09-29T05:09:06.681Z</v>
+      </c>
+    </row>
+    <row r="16" xml:space="preserve">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="str">
+        <v>All</v>
+      </c>
+      <c r="C16" t="str">
+        <v>All</v>
+      </c>
+      <c r="D16" t="str">
+        <v>give me details on implementing an MYP interdisciplinary unit</v>
+      </c>
+      <c r="E16" t="str" xml:space="preserve">
+        <v xml:space="preserve">Implementing an MYP interdisciplinary unit involves several key steps to ensure meaningful integration of disciplines and rigorous student learning:
+Purpose and Inquiry: Begin by establishing a clear, meaningful purpose for the interdisciplinary unit that aligns with the MYP philosophy and requirements. This includes identifying a real-world issue or challenge that benefits from integrating multiple disciplines. Teachers collaboratively decide on the driving questions and the product or outcome students will create, ensuring the integration is purposeful and not superficial 12.
+Planning: Use the MYP interdisciplinary unit planner, a stand-alone document designed to organize interdisciplinary teaching and learning. The planner supports teamwork and collaboration among teachers from different disciplines. Teachers select key and related concepts, global contexts, and inquiry questions (factual, conceptual, and debatable) that frame the unit 13.
+Collaboration and Reflection: Teachers work collaboratively to develop the unit plan, discussing probing questions to deepen understanding of the interdisciplinary learning process. Reviewing example unit plans at different development levels can help refine the quality of planning over time 24.
+Assessment: Develop assessment tasks using MYP interdisciplinary criteria, focusing on integration of disciplines and ATL skills. Employ diverse strategies such as observations, student journals, and portfolio analysis to collect evidence of student learning. Collaboration among teachers in assessment is important to leverage disciplinary expertise 2.
+Implementation: Deliver the unit with an emphasis on inquiry-based, concept-driven learning, ensuring students understand the purpose of integration and how different disciplines contribute to addressing the real-world issue 52.
+Support and Resources: Teachers are encouraged to use IB eAssessment materials and teacher support materials (TSM) as practical guides for planning and teaching interdisciplinary units 24.
+Following these steps helps schools create interdisciplinary units that are meaningful, rigorous, and aligned with the MYP framework, fostering students' ability to integrate knowledge and skills across disciplines 51324.
+1Interdisciplinary teaching and learning in the MYP (for use from September 2021/January 2022)_interdisciplinary-teaching-and-learning-in-the-myp-guide-en_1700f2b5-ce51-4dae-b272-c75303fca437.xml_122Interdisciplinary teaching and learning in the MYP (for use from September 2021/January 2022)_interdisciplinary-teaching-and-learning-in-the-myp-guide-en_1700f2b5-ce51-4dae-b272-c75303fca437.xml_203Interdisciplinary teaching and learning in the MYP (for use from September 2021/January 2022)_interdisciplinary-teaching-and-learning-in-the-myp-guide-en_1700f2b5-ce51-4dae-b272-c75303fca437.xml_114Interdisciplinary teaching and learning in the MYP teacher support material_interdisciplinary-teaching-and-learning-in-the-myp-tsm-en_8037eec6-6d4a-465c-aed4-04ebe1484ed2.xml_15Interdisciplinary teaching and learning in the MYP (for use from September 2021/January 2022)_interdisciplinary-teaching-and-learning-in-the-myp-guide-en_1700f2b5-ce51-4dae-b272-c75303fca437.xml_1</v>
+      </c>
+      <c r="F16" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G16" t="str">
+        <v>2026-09-29T05:09:27.706Z</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="str">
+        <v>All</v>
+      </c>
+      <c r="C17" t="str">
+        <v>All</v>
+      </c>
+      <c r="D17" t="str">
+        <v>when is MYP resources expected to be available on IB Exchange?</v>
+      </c>
+      <c r="E17" t="str">
+        <v>The retrieved documents do not provide specific information regarding the expected availability date of MYP resources on IB Exchange. For the most accurate and up-to-date details, it is recommended to consult the IB Programme Resource Centre or contact your IB regional office directly.</v>
+      </c>
+      <c r="F17" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G17" t="str">
+        <v>2026-09-29T05:09:43.059Z</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="str">
+        <v>All</v>
+      </c>
+      <c r="C18" t="str">
+        <v>All</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Why can't you process these requests? What did I do wrong?</v>
+      </c>
+      <c r="E18" t="str">
+        <v>You haven't done anything wrong. The information you provided relates mostly to AI and its impact on learning, inquiry, and knowledge, but it doesn't include details about the IB's policies or procedures regarding processing requests or submissions. Therefore, I don't have the necessary IB-specific context to answer questions about why certain IB requests might not be processed. For questions about IB administrative processes or technical issues, please contact your IB coordinator or the official IB support channels for assistance.</v>
+      </c>
+      <c r="F18" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G18" t="str">
+        <v>2026-09-29T05:09:54.640Z</v>
+      </c>
+    </row>
+    <row r="19" xml:space="preserve">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="str">
+        <v>All</v>
+      </c>
+      <c r="C19" t="str">
+        <v>All</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Where can I get sample papers for MYP1 to MYP4?</v>
+      </c>
+      <c r="E19" t="str" xml:space="preserve">
+        <v xml:space="preserve">Sample papers for MYP mathematics and other subjects for MYP1 to MYP4 can be accessed through the IB's Programme Resource Centre (PRC) available on My IB. Specifically, you can find teaching materials and teacher support materials which include examples and sample questions to guide your planning. For mathematics, the teacher support material provides examples applying MYP mathematics suggested by schools worldwide, which can be helpful for preparing assessment tasks for various criteria 1.
+1Mathematics: Frequently asked questions from the webinar “How to help your students thrive during the MYP mathematics eAssessment”_m_5_mathm_faq_2403_1_e.pdf_7</v>
+      </c>
+      <c r="F19" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G19" t="str">
+        <v>2026-09-29T05:10:06.659Z</v>
+      </c>
+    </row>
+    <row r="20" xml:space="preserve">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="str">
+        <v>All</v>
+      </c>
+      <c r="C20" t="str">
+        <v>All</v>
+      </c>
+      <c r="D20" t="str">
+        <v>WOuld you like to tell me more about MYP language and literature key topics/themes that are covered in MYP 4?</v>
+      </c>
+      <c r="E20" t="str" xml:space="preserve">
+        <v xml:space="preserve">In MYP Language and Literature, including MYP 4, the curriculum emphasizes developing students' appreciation and understanding of language and literature through key concepts such as communication, connections, creativity, and perspective. These concepts are explored in greater depth as students progress, with related discipline-specific concepts introduced to suit their academic development stage.
+The course encourages the development of six interrelated skill areas: listening, speaking, reading, writing, viewing, and presenting. It promotes analytical and organizational skills in creative, personal, and imaginative ways, fostering intercultural understanding and engagement at local, national, and global levels.
+While there are no prescribed texts, teachers select a broad range of literary and non-literary texts that suit students' interests and needs, broaden their experiences, enhance historical and intercultural understanding, and model effective communication across diverse audiences and purposes. The curriculum is flexible and culturally sensitive, supporting international-mindedness.
+These elements prepare students for the Diploma Programme studies in language and literature, ensuring a smooth transition and continued development of linguistic and literary skills 12345.
+1Language A: language and literature guide_language-a-language-and-literature-guide-first-assessment-20-en_45a3922b-b147-478c-9f00-78cbf1fea859.xml_102Language A: literature guide_language-a-literature-guide-first-assessment-2021-en_f1795501-4f95-400c-960c-6c4b91a12e25.xml_103Language A: language and literature guide_language-a-language-and-literature-guide-first-assessment-20-en_45a3922b-b147-478c-9f00-78cbf1fea859.xml_114Language A: literature guide_language-a-literature-guide-first-assessment-2021-en_f1795501-4f95-400c-960c-6c4b91a12e25.xml_115Language and literature guide (for use from September 2014/January 2015)_m_1_langa_guu_1405_8_e.pdf_36</v>
+      </c>
+      <c r="F20" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G20" t="str">
+        <v>2026-09-29T05:10:24.964Z</v>
+      </c>
+    </row>
+    <row r="21" xml:space="preserve">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="str">
+        <v>All</v>
+      </c>
+      <c r="C21" t="str">
+        <v>All</v>
+      </c>
+      <c r="D21" t="str">
+        <v>math summative assessment</v>
+      </c>
+      <c r="E21" t="str" xml:space="preserve">
+        <v xml:space="preserve">In the MYP, mathematics summative assessments are designed to evaluate student achievement based on specific subject-group assessment criteria, which include:
+Criterion A: Knowing and understanding
+Criterion B: Investigating patterns
+Criterion C: Communicating
+Criterion D: Applying mathematics in real-life contexts
+Each criterion is scored with a maximum of 8 marks, and assessments are structured to allow students to demonstrate their skills and understanding across these areas 1.
+Summative assessments are integral to the learning process and should be aligned with subject-group objectives, providing authentic opportunities for students to show their knowledge and skills. They can be designed as a single task assessing multiple criteria or multiple related tasks assessing different criteria, with increasing complexity as students progress through the MYP years 23.
+For external verification, MYP students may take optional on-screen examinations (eAssessment), which follow an examination blueprint ensuring consistency and alignment with the assessment criteria. These eAssessments simulate classroom internal assessments and provide a balanced measure of student achievement 1.
+1Mathematics guide (for use from September 2020/January 2021)_mathematics-guide-for-use-from-september-2020january-2021-en_f972b695-a0a4-43b9-a744-dfce17c03b9f.xml_152MYP: From principles into practice (Updated 2022 for use with the latest Programme standards and practices)_m_0_mypxx_guu_1405_10_e.pdf_713Further guidance for developing MYP assessed curriculum_m_0_mypxx_fcl_1409_3b_e.pdf_3</v>
+      </c>
+      <c r="F21" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G21" t="str">
+        <v>2026-09-29T05:10:39.460Z</v>
+      </c>
+    </row>
+    <row r="22" xml:space="preserve">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="str">
+        <v>All</v>
+      </c>
+      <c r="C22" t="str">
+        <v>All</v>
+      </c>
+      <c r="D22" t="str" xml:space="preserve">
+        <v xml:space="preserve">Subject (optional): Request for examples of high-scoring MYP Personal Projects (Japanese)_x000d__x000d_
+Thank you for your continued support._x000d__x000d_
+My name is Naoki Kobayashi, MYP Coordinator at Kaichi Nozomi Secondary School. We had the pleasure of exchanging business cards at the IBAJ conference in April._x000d__x000d_
+I am writing to kindly ask whether you might be willing to share examples of how MYP Personal Projects written in Japanese are assessed, particularly those that have achieved the highest levels._x000d__x000d_
+Our school has been implementing the Personal Project (PP) for the past three years; however, the highest score we have awarded in both Japanese and English to date is 5. In an effort to better understand this, I have reached out to other MYP Coordinators to inquire whether they could anonymously share examples of projects that received a 7. Several colleagues indicated that while some students have achieved a 7 in English-language PPs, scores for Japanese-language PPs tend to remain at 5 or 6. They also noted that, despite providing comparable levels of support and instruction in both languages, improving outcomes in Japanese has been a persistent challenge._x000d__x000d_
+With regard to English-language PPs, we have been referring to the sample materials available in the PRC section of MyIB to guide our teaching and assessment. Nevertheless, we continue to face difficulties in achieving higher levels of student performance._x000d__x000d_
+We would be most grateful if you could share any relevant examples or insights you may have. Thank you very much for considering this request._x000d__x000d_
+Yours sincerely,_x000d__x000d_
+Naoki Kobayashi</v>
+      </c>
+      <c r="E22" t="str">
+        <v/>
+      </c>
+      <c r="F22" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G22" t="str">
+        <v>2026-09-29T05:11:28.140Z</v>
+      </c>
+    </row>
+    <row r="23" xml:space="preserve">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="str">
+        <v>All</v>
+      </c>
+      <c r="C23" t="str">
+        <v>All</v>
+      </c>
+      <c r="D23" t="str">
+        <v>called to ask if they can have an IB elective class added to their curriculum. The class would not count towards the 8 disciplines for the MYP, and would not fall under any specific subject. I advised I will escalate to curriculum.</v>
+      </c>
+      <c r="E23" t="str" xml:space="preserve">
+        <v xml:space="preserve">In the MYP, students are generally expected to study courses from at least six subject groups concurrently in years 4 and 5, including language and literature, language acquisition, individuals and societies, sciences, mathematics, and one additional subject group (arts, design, or physical and health education) 1. While schools have flexibility to combine subject groups or offer electives, any additional courses outside the core subject groups typically do not count towards the required eight disciplines for the MYP certificate 12.
+Offering an IB elective class that does not fall under a specific subject group and does not contribute to the core MYP subject requirements is possible, but it would be considered outside the formal MYP subject-group framework. Such an elective would be an addition to the curriculum rather than part of the assessed MYP disciplines. It is appropriate to escalate this request to curriculum coordinators to ensure alignment with IB programme requirements and school policies 12.
+1MYP: From principles into practice 2014 (For candidate schools following the 2014 Programme standards and practices authorization process)_m_0_mypxx_guu_2209_1_e.pdf_422Interdisciplinary teaching and learning in the MYP (for use from September 2021/January 2022)_interdisciplinary-teaching-and-learning-in-the-myp-guide-en_1700f2b5-ce51-4dae-b272-c75303fca437.xml_3</v>
+      </c>
+      <c r="F23" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G23" t="str">
+        <v>2026-09-29T05:11:42.621Z</v>
+      </c>
+    </row>
+    <row r="24" xml:space="preserve">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="str">
+        <v>All</v>
+      </c>
+      <c r="C24" t="str">
+        <v>All</v>
+      </c>
+      <c r="D24" t="str">
+        <v>ATL framework</v>
+      </c>
+      <c r="E24" t="str" xml:space="preserve">
+        <v xml:space="preserve">The Approaches to Learning (ATL) framework in the MYP is a central element designed to develop students' learning skills across all subjects and years. It consists of five broad categories of ATL skills that support students in becoming effective, independent learners. These skills are both subject-specific and general, inclusive of "soft skills," and aligned with the IB learner profile values. Schools are expected to plan for the vertical (across years) and horizontal (across subjects) articulation of ATL skills to ensure meaningful progression and coordination of students' learning experiences. The framework is intended to be integral to unit planning and owned by students to promote lifelong learning abilities. While schools are not required to report on all ATL skills formally, meaningful feedback and self-evaluation of ATL skill development are encouraged to enhance student growth. Collaborative planning among teachers and structured time for horizontal planning are important to support the effective implementation of ATL skills in the curriculum. The ATL planning can be organized flexibly, using charts or other documents, and may be informed by external standards or frameworks to scaffold skill development progressively throughout the MYP 12345.
+1Further guidance for developing ATL in the MYP_m_0_mypxx_fcl_1409_1a_e.pdf_12Further guidance for developing ATL in the MYP_m_0_mypxx_fcl_1409_1a_e.pdf_33Further guidance for developing ATL in the MYP_m_0_mypxx_fcl_1409_1a_e.pdf_44Further guidance for developing ATL in the MYP_m_0_mypxx_fcl_1409_1a_e.pdf_85Further guidance for developing ATL in the MYP_m_0_mypxx_fcl_1409_1a_e.pdf_6</v>
+      </c>
+      <c r="F24" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G24" t="str">
+        <v>2026-09-29T05:11:57.813Z</v>
+      </c>
+    </row>
+    <row r="25" xml:space="preserve">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="str">
+        <v>All</v>
+      </c>
+      <c r="C25" t="str">
+        <v>All</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Can you a frame a question where all 4 programms are interrelated? frame any 2</v>
+      </c>
+      <c r="E25" t="str" xml:space="preserve">
+        <v xml:space="preserve">Here are two example questions that interrelate all four IB programmes (PYP, MYP, DP, and CP) by focusing on connected, interdisciplinary learning and global contexts:
+How can the concept of sustainability be explored and addressed across different disciplines and IB programmes, from early inquiry in the PYP through interdisciplinary projects in the MYP, to advanced research in the DP and career-related applications in the CP?
+In what ways can international-mindedness and global citizenship be developed through the transdisciplinary themes of the PYP, conceptual and connected curriculum in the MYP, theory of knowledge and extended essay investigations in the DP, and reflective projects in the CP?
+These questions emphasize the continuum of learning across programmes, highlighting the increasing disciplinary complexity and integration while maintaining a connected and holistic educational experience 1234.
+1Interdisciplinary teaching and learning in the MYP (for use from September 2021/January 2022)_interdisciplinary-teaching-and-learning-in-the-myp-guide-en_1700f2b5-ce51-4dae-b272-c75303fca437.xml_32Interdisciplinary teaching and learning in the MYP (for use from September 2021/January 2022)_interdisciplinary-teaching-and-learning-in-the-myp-guide-en_1700f2b5-ce51-4dae-b272-c75303fca437.xml_43Interdisciplinary teaching and learning in the MYP (for use from September 2021/January 2022)_interdisciplinary-teaching-and-learning-in-the-myp-guide-en_1700f2b5-ce51-4dae-b272-c75303fca437.xml_54What is an IB education?_what-is-an-ib-education-en_148279a4-dd5d-4552-bd1c-187c8442d91c.xml_3</v>
+      </c>
+      <c r="F25" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G25" t="str">
+        <v>2026-09-29T05:12:13.228Z</v>
+      </c>
+    </row>
+    <row r="26" xml:space="preserve">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="str">
+        <v>All</v>
+      </c>
+      <c r="C26" t="str">
+        <v>All</v>
+      </c>
+      <c r="D26" t="str">
+        <v>what are the requirements to receive your CP certificate</v>
+      </c>
+      <c r="E26" t="str" xml:space="preserve">
+        <v xml:space="preserve">To receive the IB Career-related Programme (CP) certificate, a student must satisfactorily complete several requirements including:
+Completion of the specified career-related study.
+Achieving a grade of 3 or higher in at least two Diploma Programme (DP) courses.
+Earning a grade of D or higher on the reflective project.
+Meeting the requirements for personal and professional skills, service learning (minimum 50 hours), and language development (minimum 50 hours).
+Not receiving any penalties for academic misconduct.
+Upon meeting these conditions, students are awarded the IB CP Certificate along with a statement of results detailing their achievements in DP courses, the reflective project, and the status of CP core completion 123.
+1Career-related Programme Assessment procedures 2026_cp-assessment-procedures-2026-en_bd9462b2-fc3e-40db-be74-b80152ab95e2.xml_52Letter to accompany university application Career-related Programme, 2025_d_x_carec_grad_2409_2_e.pdf_23Career-related Programme Assessment procedures 2026_cp-assessment-procedures-2026-en_bd9462b2-fc3e-40db-be74-b80152ab95e2.xml_10</v>
+      </c>
+      <c r="F26" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G26" t="str">
+        <v>2026-09-29T05:12:28.272Z</v>
+      </c>
+    </row>
+    <row r="27" xml:space="preserve">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="str">
+        <v>All</v>
+      </c>
+      <c r="C27" t="str">
+        <v>All</v>
+      </c>
+      <c r="D27" t="str">
+        <v>what does sustained engagement over the duration of the Cp mean in practical terms</v>
+      </c>
+      <c r="E27" t="str" xml:space="preserve">
+        <v xml:space="preserve">In practical terms, "sustained engagement over the duration of the CP" means that students consistently participate and remain actively involved in all components of the Career-related Programme throughout the entire period of study (typically ages 16 to 19). This includes continuous commitment to their career-related study, Diploma Programme courses, the CP core components (such as the reflective project, language development, service learning, and personal and professional skills), and related assessments. Sustained engagement requires students to demonstrate ongoing effort, time management, and development of skills and knowledge rather than sporadic or minimal involvement, ensuring they meet the learning outcomes and requirements of the CP framework 12.
+1Community engagement guide (first teaching 2025)_cp-community-engagement-guide-2025-en_91e189b0-9664-4328-b3eb-dfe61b281fb9.xml_12Career-related Programme Assessment procedures 2026_cp-assessment-procedures-2026-en_bd9462b2-fc3e-40db-be74-b80152ab95e2.xml_2</v>
+      </c>
+      <c r="F27" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G27" t="str">
+        <v>2026-09-29T05:12:43.020Z</v>
+      </c>
+    </row>
+    <row r="28" xml:space="preserve">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" t="str">
+        <v>All</v>
+      </c>
+      <c r="C28" t="str">
+        <v>All</v>
+      </c>
+      <c r="D28" t="str">
+        <v>What are the differences between IBDP and IBCP?</v>
+      </c>
+      <c r="E28" t="str" xml:space="preserve">
+        <v xml:space="preserve">The International Baccalaureate Diploma Programme (IBDP) and the Career-related Programme (IBCP) differ primarily in focus and structure:
+IBDP is a two-year academic programme for students aged 16-19 that offers a broad and challenging curriculum across six subject groups. It emphasizes interdisciplinary understanding, critical thinking, and preparation for university-level study. Students take courses at standard or higher level, complete core components like the Extended Essay and Theory of Knowledge, and aim for the full IB Diploma 12.
+IBCP is designed for students aged 16-19 who want to combine academic study with career-related learning. It includes at least two Diploma Programme courses, a career-related study (which is not offered or awarded by the IB but must meet IB criteria), and a distinctive CP core that develops personal and professional skills, service learning, language development, and a reflective project. The CP prepares students for higher education, apprenticeships, or employment by integrating applied knowledge and practical skills with academic rigor 324.
+In summary, the IBDP is more academic and broad-based, while the IBCP offers a flexible framework combining academic courses with career-related education and skills development.
+1Research report— Postsecondary outcomes of International Baccalaureate Diploma Programme graduates in the United States (2024)_g_0_ibres_sur-ir_2406_1a_e.pdf_22Research report— Postsecondary outcomes of International Baccalaureate Career-related Programme graduates in the United States (2024)_g_0_ibres_sur-ir_2406_1_e.pdf_23Letter to accompany university application Career-related Programme, 2025_d_x_carec_grad_2409_2_e.pdf_14Overview of the Career-related Programme_d_0_carec_amo-16_1512_1_e.pdf_3</v>
+      </c>
+      <c r="F28" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G28" t="str">
+        <v>2026-09-29T05:12:57.746Z</v>
+      </c>
+    </row>
+    <row r="29" xml:space="preserve">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" t="str">
+        <v>All</v>
+      </c>
+      <c r="C29" t="str">
+        <v>All</v>
+      </c>
+      <c r="D29" t="str">
+        <v>what planner do i use for the PYP exhibition AF</v>
+      </c>
+      <c r="E29" t="str" xml:space="preserve">
+        <v xml:space="preserve">For the PYP exhibition, you use the PYP planner as outlined in Making the PYP Happen: A Curriculum Framework for International Primary Education (2009). Each exhibition must be documented on a PYP planner if it is included within the programme of inquiry. However, schools have the flexibility to implement the exhibition outside of the programme of inquiry, in which case a PYP planner is not required. This flexibility allows schools to adapt the exhibition to their context while supporting student agency and inquiry 123.
+1Coordinator’s handbook 2013 - 2014_p_0_pypxx_coh_1308_1_e.pdf_392PYP: From principles into practice FAQs_p_0_pypxx_faq_2008_4_e.pdf_63The Learner in the enhanced PYP_p_0_pypxx_amo_1711_1_e.pdf_6</v>
+      </c>
+      <c r="F29" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G29" t="str">
+        <v>2026-09-29T05:13:10.085Z</v>
+      </c>
+    </row>
+    <row r="30" xml:space="preserve">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" t="str">
+        <v>All</v>
+      </c>
+      <c r="C30" t="str">
+        <v>All</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Nothing about age 3-6 learners? We have a lot of bilingual multilingual learners ST</v>
+      </c>
+      <c r="E30" t="str" xml:space="preserve">
+        <v xml:space="preserve">_x001b_[2mexpect(_x001b_[22m_x001b_[31mreceived_x001b_[39m_x001b_[2m)._x001b_[22mtoBeGreaterThan_x001b_[2m(_x001b_[22m_x001b_[32mexpected_x001b_[39m_x001b_[2m)_x001b_[22m
+Expected: &gt; _x001b_[32m27_x001b_[39m
+Received:   _x001b_[31m27_x001b_[39m
+Call Log:
+- Timeout 180000ms exceeded while waiting on the predicate</v>
+      </c>
+      <c r="F30" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="G30" t="str">
+        <v>2026-09-29T05:16:14.087Z</v>
+      </c>
+    </row>
+    <row r="31" xml:space="preserve">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" t="str">
+        <v>All</v>
+      </c>
+      <c r="C31" t="str">
+        <v>All</v>
+      </c>
+      <c r="D31" t="str">
+        <v>there are 3 strands in PSPE ST</v>
+      </c>
+      <c r="E31" t="str" xml:space="preserve">
+        <v xml:space="preserve">Yes, the three strands in the PYP Personal, Social, and Physical Education (PSPE) are Identity, Active Living, and Interactions. These strands organize the learning continuums and provide a framework for developing conceptual understandings and learner outcomes across the phases of the programme 1.
+1PSPE development report: Second report for teachers (April 2022)_p_0_pypxx_sur_2204_3p_e.pdf_6</v>
+      </c>
+      <c r="F31" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G31" t="str">
+        <v>2026-09-29T05:16:28.737Z</v>
+      </c>
+    </row>
+    <row r="32" xml:space="preserve">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" t="str">
+        <v>All</v>
+      </c>
+      <c r="C32" t="str">
+        <v>All</v>
+      </c>
+      <c r="D32" t="str">
+        <v>are the approaches to teaching the same in the PYP and MYP ST</v>
+      </c>
+      <c r="E32" t="str" xml:space="preserve">
+        <v xml:space="preserve">The approaches to teaching in the PYP and MYP share some underlying principles but are tailored to suit the developmental stages and specific aims of each programme. In the MYP, teaching styles are evolving from traditional subject-focused transmission to more skills-based, process-oriented methods that promote student self-regulation and engagement. This includes shared regulation between teacher and students and process-oriented instruction that supports independent learning and metacognitive skills development 12.
+In the PYP, teaching approaches emphasize transdisciplinary learning and designing curricula that integrate PSPE with other subjects, focusing on holistic development including play, relationships, and symbolic exploration in early years. The PYP also highlights the role of the teacher as a curriculum designer and uses IB approaches to teaching to support this design process 34.
+Therefore, while both programmes value student agency, inquiry, and skill development, the MYP has a stronger focus on transitioning students towards more andragogical, self-regulated learning styles as they mature, whereas the PYP emphasizes early holistic and transdisciplinary learning experiences 12.
+1Approaches to learning and approaches to teaching in the Middle Years Programme_approaches-to-learning-and-approaches-to-teaching-in-the-mid-en_af9646cb-da0c-4a76-bc1d-4c127a5b7744.xml_192Approaches to learning and approaches to teaching in the Middle Years Programme_approaches-to-learning-and-approaches-to-teaching-in-the-mid-en_af9646cb-da0c-4a76-bc1d-4c127a5b7744.xml_183PSPE development report: First report for teachers (April 2021)_p_0_pypxx_sur_2104_1p_e.pdf_54PSPE development report: First report for teachers (April 2021)_p_0_pypxx_sur_2104_1p_e.pdf_6</v>
+      </c>
+      <c r="F32" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G32" t="str">
+        <v>2026-09-29T05:16:44.219Z</v>
+      </c>
+    </row>
+    <row r="33" xml:space="preserve">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33" t="str">
+        <v>All</v>
+      </c>
+      <c r="C33" t="str">
+        <v>All</v>
+      </c>
+      <c r="D33" t="str">
+        <v>can enviromental sciene be an interdisciplinary subject</v>
+      </c>
+      <c r="E33" t="str" xml:space="preserve">
+        <v xml:space="preserve">Yes, Environmental Science can be an interdisciplinary subject. It combines methodologies and techniques from both experimental sciences and human sciences, reflecting its interdisciplinary nature. This allows students to explore ecological concepts, environmental laws, economics, and ethical considerations in a connected way. For example, students can study environmental issues using both qualitative and quantitative methods, investigate local or global problems, and apply knowledge from various disciplines to understand and address sustainability challenges 123.
+1Environmental systems and societies teacher support material_environmental-systems-teacher-support-material-en_c1c4de2e-8fe2-4f21-afb9-7531d9d1c45c.xml_32Environmental systems and societies teacher support material_environmental-systems-teacher-support-material-en_c1c4de2e-8fe2-4f21-afb9-7531d9d1c45c.xml_113Environmental systems and societies teacher support material_environmental-systems-teacher-support-material-en_c1c4de2e-8fe2-4f21-afb9-7531d9d1c45c.xml_23</v>
+      </c>
+      <c r="F33" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G33" t="str">
+        <v>2026-09-29T05:16:58.912Z</v>
+      </c>
+    </row>
+    <row r="34" xml:space="preserve">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34" t="str">
+        <v>All</v>
+      </c>
+      <c r="C34" t="str">
+        <v>All</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Are there any subject guides for the MYP beta</v>
+      </c>
+      <c r="E34" t="str" xml:space="preserve">
+        <v xml:space="preserve">Yes, there are subject guides and enhanced curriculum content available as part of the Enhancing the MYP BETA trial. The trial provides updated curriculum guidance on unit planning and other components to support schools participating in the beta phase. Resources such as the Enhancing the MYP BETA trial website contain curriculum content and guidance, and workshops are offered to help educators engage with enhanced unit planning, curriculum design, and implementation strategies 12.
+1Enhancing the MYP: Making the MYP better for all students, teachers and school communities_enhancing-the-myp-making-the-myp-better-for-all-students-tea-en_a0dd97db-7c45-4106-a1bd-d6a515abcc9b.xml_22Middle Years Programme updates, May 2025_m_g_mypxx_con_2505_1_e.pdf_2</v>
+      </c>
+      <c r="F34" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G34" t="str">
+        <v>2026-09-29T05:17:10.962Z</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35" t="str">
+        <v>All</v>
+      </c>
+      <c r="C35" t="str">
+        <v>All</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Is making mistakes in grammar in French B tested in criterion A ?</v>
+      </c>
+      <c r="E35" t="str">
+        <v>Yes, in French B, making mistakes in grammar is considered under Criterion A, which evaluates the student's linguistic competence. This includes vocabulary, grammatical structures, language accuracy, pronunciation, and intonation. Errors that interfere with communication, such as grammatical mistakes that make sentences incoherent or difficult to understand, affect the Criterion A assessment. However, minor errors that do not hinder understanding may have less impact on the mark .</v>
+      </c>
+      <c r="F35" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G35" t="str">
+        <v>2026-09-29T05:17:32.418Z</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36" t="str">
+        <v>All</v>
+      </c>
+      <c r="C36" t="str">
+        <v>All</v>
+      </c>
+      <c r="D36" t="str">
+        <v>is it mandatory to teach design?</v>
+      </c>
+      <c r="E36" t="str">
+        <v>I'm sorry, I'm unable to process this request.</v>
+      </c>
+      <c r="F36" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G36" t="str">
+        <v>2026-09-29T05:17:44.479Z</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37" t="str">
+        <v>All</v>
+      </c>
+      <c r="C37" t="str">
+        <v>All</v>
+      </c>
+      <c r="D37" t="str">
+        <v>do kids have to do teh eassessmsnt in myp 5</v>
+      </c>
+      <c r="E37" t="str">
+        <v>I'm sorry, I'm unable to process this request.</v>
+      </c>
+      <c r="F37" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G37" t="str">
+        <v>2026-09-29T05:17:59.801Z</v>
+      </c>
+    </row>
+    <row r="38" xml:space="preserve">
+      <c r="A38">
+        <v>37</v>
+      </c>
+      <c r="B38" t="str">
+        <v>All</v>
+      </c>
+      <c r="C38" t="str">
+        <v>All</v>
+      </c>
+      <c r="D38" t="str">
+        <v>can a student who has been in Lang Lit in MYP do Lang B in the same language in DP if they do not have the level for the Lang Lit in DP?</v>
+      </c>
+      <c r="E38" t="str" xml:space="preserve">
+        <v xml:space="preserve">A student who has studied Language and Literature (Lang Lit) in the MYP but does not have the required level for Language and Literature in the Diploma Programme (DP) may consider taking Language B in the same language in the DP, provided their linguistic proficiency aligns better with Language B requirements. The MYP Language acquisition guide recommends that students achieve at least Phase 5 or Phase 6 in Language acquisition before progressing to DP studies in language and literature, and sometimes it is suggested that students have some MYP Language and Literature experience for a smoother transition. Ultimately, the choice between Language and Literature and Language B in the DP depends on the student’s language proficiency and should be made in consultation with teachers and coordinators to ensure an appropriate match to the student's skills and educational goals 12.
+1Language A: language and literature guide_d_1_alanl_gui_2507_1_e.pdf_162Language A: literature guide_d_1_alite_gui_2507_1_e.pdf_15</v>
+      </c>
+      <c r="F38" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G38" t="str">
+        <v>2026-09-29T05:18:14.936Z</v>
+      </c>
+    </row>
+    <row r="39" xml:space="preserve">
+      <c r="A39">
+        <v>38</v>
+      </c>
+      <c r="B39" t="str">
+        <v>All</v>
+      </c>
+      <c r="C39" t="str">
+        <v>All</v>
+      </c>
+      <c r="D39" t="str">
+        <v>When is the IBCP Refelctive Project turned into the IB?</v>
+      </c>
+      <c r="E39" t="str" xml:space="preserve">
+        <v xml:space="preserve">The IB Career-related Programme (IBCP) Reflective Project is submitted towards the end of the Career-related Programme. Students work on it over an extended period, and it is expected that they devote a minimum of 50 hours to its completion. After the school assesses the Reflective Project, a sample is sent electronically to the IB for external moderation. The submission must be in one of the IB working languages (English, Spanish, or French), and live links are not permitted. The final submission includes the written essay (or essay plus an additional format) and the Reflections on Planning and Progress Form (RPPF) 123.
+1Reflective project guide (last assessment 2026)_d_0_carec_gui-16_1512_2r_e.pdf_102Reflective project teacher support material (last assessment 2026)_cp-reflective-project-tsm-2015-en_f954c3a4-289c-403e-8d7e-33f490aba326.xml_13Additional guidance for the reflective project (last assessment 2026)_d_0_carec_amo_1604_1_e.pdf_4</v>
+      </c>
+      <c r="F39" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G39" t="str">
+        <v>2026-09-29T05:18:27.068Z</v>
+      </c>
+    </row>
+    <row r="40" xml:space="preserve">
+      <c r="A40">
+        <v>39</v>
+      </c>
+      <c r="B40" t="str">
+        <v>All</v>
+      </c>
+      <c r="C40" t="str">
+        <v>All</v>
+      </c>
+      <c r="D40" t="str">
+        <v>hiw many hours are required</v>
+      </c>
+      <c r="E40" t="str" xml:space="preserve">
+        <v xml:space="preserve">Students are expected to devote a minimum of 50 hours to complete the IB Career-related Programme Reflective Project over an extended period of time 123.
+1Reflective project guide (first teaching 2025)_cp-reflective-project-guide-2025-en_56cec644-bd5f-4ba1-a167-d7996151afc2.xml_72Reflective project guide (last assessment 2026)_d_0_carec_gui-16_1512_2r_e.pdf_73Reflective project guide (last assessment 2026)_d_0_carec_gui-16_1512_2r_e.pdf_6</v>
+      </c>
+      <c r="F40" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G40" t="str">
+        <v>2026-09-29T05:18:39.389Z</v>
+      </c>
+    </row>
+    <row r="41" xml:space="preserve">
+      <c r="A41">
+        <v>40</v>
+      </c>
+      <c r="B41" t="str">
+        <v>All</v>
+      </c>
+      <c r="C41" t="str">
+        <v>All</v>
+      </c>
+      <c r="D41" t="str">
+        <v>Tell me about assessing the IBCP core components</v>
+      </c>
+      <c r="E41" t="str" xml:space="preserve">
+        <v xml:space="preserve">The assessment of the IB Career-related Programme (IBCP) core components involves evaluating the Reflective Project, which is externally assessed and focuses on an ethical dilemma related to the student's career-related studies. The assessment criteria include:
+Criterion A: Focus on the ethical dilemma — assessing how well the ethical dilemma is identified and explored from different perspectives and contexts.
+Criterion B: Knowledge and understanding through research — evaluating the use of research to develop understanding of the ethical dilemma and its impacts.
+Criterion C: Critical thinking — analyzing and synthesizing research to justify a personal position considering implications for various contexts and groups.
+Criterion D: Communication of ideas — assessing clarity, organization, terminology, and structure in communicating ideas.
+Criterion E: Reflective practice — evaluating the planning, research, and implementation of reflective practices during the project.
+The Reflective Project is externally moderated, and supervisors do not assign marks but may provide predicted grades based on qualitative grade descriptors. These descriptors guide understanding of the academic expectations and help in setting grade boundaries during moderation. Schools must also review and evaluate the delivery of all core components regularly to ensure relevance and integration, as part of ongoing quality assurance and programme evaluation processes 1.
+1Reflective project guide (first teaching 2025)_cp-reflective-project-guide-2025-en_56cec644-bd5f-4ba1-a167-d7996151afc2.xml_26</v>
+      </c>
+      <c r="F41" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G41" t="str">
+        <v>2026-09-29T05:18:54.521Z</v>
+      </c>
+    </row>
+    <row r="42" xml:space="preserve">
+      <c r="A42">
+        <v>41</v>
+      </c>
+      <c r="B42" t="str">
+        <v>All</v>
+      </c>
+      <c r="C42" t="str">
+        <v>All</v>
+      </c>
+      <c r="D42" t="str">
+        <v>is a language B required for the CP?</v>
+      </c>
+      <c r="E42" t="str" xml:space="preserve">
+        <v xml:space="preserve">No, a Language B course is not specifically required for the IB Career-related Programme (CP). However, language development is a core component of the CP, ensuring that all students have access to and are exposed to an additional language. Students are encouraged to begin or extend the study of a language other than their best language to develop their linguistic and communicative abilities. A minimum of 50 hours is expected to be devoted to language development as part of the CP core, but this does not mandate a Language B course specifically 123.
+1Letter to accompany university application Career-related Programme, 2025_d_x_carec_grad_2409_2_e.pdf_22Career-related Programme Assessment procedures 2026_cp-assessment-procedures-2026-en_bd9462b2-fc3e-40db-be74-b80152ab95e2.xml_43Career-related Programme Assessment procedures 2026_cp-assessment-procedures-2026-en_bd9462b2-fc3e-40db-be74-b80152ab95e2.xml_5</v>
+      </c>
+      <c r="F42" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G42" t="str">
+        <v>2026-09-29T05:19:06.351Z</v>
+      </c>
+    </row>
+    <row r="43" xml:space="preserve">
+      <c r="A43">
+        <v>42</v>
+      </c>
+      <c r="B43" t="str">
+        <v>All</v>
+      </c>
+      <c r="C43" t="str">
+        <v>All</v>
+      </c>
+      <c r="D43" t="str">
+        <v>Community Engagement hours</v>
+      </c>
+      <c r="E43" t="str" xml:space="preserve">
+        <v xml:space="preserve">Schools are expected to allocate a minimum of 30 guided hours for the Community Engagement (CE) component of the IB Career-related Programme (CP). These guided hours cover the introduction, orientation, ongoing guidance, and review points for CE. However, the total number of hours students actively engage with the community outside of guided learning is not specified, as the focus is on sustained and meaningful engagement rather than a set quantity of hours. Schools may provide additional hours beyond the minimum to support students’ aspirations for CE 1.
+1Community engagement guide (first teaching 2025)_cp-community-engagement-guide-2025-en_91e189b0-9664-4328-b3eb-dfe61b281fb9.xml_17</v>
+      </c>
+      <c r="F43" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G43" t="str">
+        <v>2026-09-29T05:19:18.575Z</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44">
+        <v>43</v>
+      </c>
+      <c r="B44" t="str">
+        <v>All</v>
+      </c>
+      <c r="C44" t="str">
+        <v>All</v>
+      </c>
+      <c r="D44" t="str">
+        <v>What kind of Language students can take in language devleopment in CP Programme</v>
+      </c>
+      <c r="E44" t="str">
+        <v>I'm sorry, I'm unable to process this request.</v>
+      </c>
+      <c r="F44" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G44" t="str">
+        <v>2026-09-29T05:19:31.069Z</v>
+      </c>
+    </row>
+    <row r="45" xml:space="preserve">
+      <c r="A45">
+        <v>44</v>
+      </c>
+      <c r="B45" t="str">
+        <v>All</v>
+      </c>
+      <c r="C45" t="str">
+        <v>All</v>
+      </c>
+      <c r="D45" t="str">
+        <v>Is there a guide for writing an assessment policy? ST</v>
+      </c>
+      <c r="E45" t="str" xml:space="preserve">
+        <v xml:space="preserve">Yes, there is guidance for schools on developing an assessment policy. Constructing and implementing an assessment policy helps schools engage meaningfully with IB assessment expectations while considering their unique context. The process involves understanding IB principles, comparing them with the school's current practices, and synthesizing these into a policy document that reflects a common understanding within the school community. The policy should include a philosophy of assessment, detail assessment practices (both formative and summative), and explain how grading, recording, and reporting are handled. It should also address timelines, workloads, and communicate assessment purposes clearly to all stakeholders. The policy must be a living document, collaboratively written, and regularly reviewed to improve practice. Schools can find this guidance in IB resources such as "Guidelines for developing a school assessment policy in the Diploma Programme" and related programme guides 123.
+1Guidelines for developing a school assessment policy in the Diploma Programme_d_0_dpyyy_ass_1101_1_e.pdf_22MYP: From principles into practice (Updated 2022 for use with the latest Programme standards and practices)_m_0_mypxx_guu_1405_10_e.pdf_383Guidelines for developing a school assessment policy in the Diploma Programme_d_0_dpyyy_ass_1101_1_e.pdf_5</v>
+      </c>
+      <c r="F45" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G45" t="str">
+        <v>2026-09-29T05:19:46.271Z</v>
+      </c>
+    </row>
+    <row r="46" xml:space="preserve">
+      <c r="A46">
+        <v>45</v>
+      </c>
+      <c r="B46" t="str">
+        <v>All</v>
+      </c>
+      <c r="C46" t="str">
+        <v>All</v>
+      </c>
+      <c r="D46" t="str" xml:space="preserve">
+        <v xml:space="preserve">I need the document: The IB learner profile AF_x000d__x000d_
+The IB learner profile represents a broad range of human capacities and responsibilities that encompass intellectual, personal, emotional, and social growth. It supports students in developing international-mindedness and taking action for positive change. Through inquiry and reflection, learners develop attributes such as being open-minded, caring, and principled, which are explored and revisited across the transdisciplinary themes and subject-spec</v>
+      </c>
+      <c r="E46" t="str">
+        <v/>
+      </c>
+      <c r="F46" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G46" t="str">
+        <v>2026-09-29T05:20:32.156Z</v>
+      </c>
+    </row>
+    <row r="47" xml:space="preserve">
+      <c r="A47">
+        <v>46</v>
+      </c>
+      <c r="B47" t="str">
+        <v>All</v>
+      </c>
+      <c r="C47" t="str">
+        <v>All</v>
+      </c>
+      <c r="D47" t="str">
+        <v>What is the difference between Maths AI and Maths AA?</v>
+      </c>
+      <c r="E47" t="str" xml:space="preserve">
+        <v xml:space="preserve">The difference between Mathematics: Applications and Interpretation (AI) and Mathematics: Analysis and Approaches (AA) lies primarily in their focus and approach:
+Mathematics: Analysis and Approaches (AA) is designed for students who enjoy developing strong mathematical thinking and fluency in constructing mathematical arguments. It includes traditional pre-university topics such as functions, trigonometry, calculus, sequences and series, and proof by induction. AA emphasizes analytical expertise and mathematical problem solving, with a strong focus on justifying and communicating mathematical arguments. It also allows the use of technology but prioritizes understanding and constructing proofs. AA is suitable for students interested in STEM fields or who enjoy abstract and theoretical mathematics 12.
+Mathematics: Applications and Interpretation (AI) focuses on the practical application of mathematics to describe the world and solve real-life problems. It emphasizes mathematical modelling and the use of technology to explore and construct models. AI includes topics like calculus and statistics but is more oriented towards applied mathematics and data interpretation. This course suits students who prefer contextual and practical mathematics, often in data-rich environments 12.
+In summary, AA is more theoretical and proof-oriented, while AI is more applied and modelling-focused, catering to different student interests and future academic or career paths .
+1Mathematics: applications and interpretation guide_mathematics-applications-and-interpretation-guide-en_f67500d4-c8e4-4d84-b3b6-26ea0c58132b.xml_62Mathematics: analysis and approaches guide_mathematics-analysis-and-approaches-guide-en_6b6db2f8-f7ce-414b-a41a-c090a26d5888.xml_6</v>
+      </c>
+      <c r="F47" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G47" t="str">
+        <v>2026-09-29T05:20:46.957Z</v>
+      </c>
+    </row>
+    <row r="48" xml:space="preserve">
+      <c r="A48">
+        <v>47</v>
+      </c>
+      <c r="B48" t="str">
+        <v>All</v>
+      </c>
+      <c r="C48" t="str">
+        <v>All</v>
+      </c>
+      <c r="D48" t="str">
+        <v>What is the MYP?</v>
+      </c>
+      <c r="E48" t="str" xml:space="preserve">
+        <v xml:space="preserve">The Middle Years Programme (MYP) is a comprehensive curriculum framework designed by the International Baccalaureate (IB) for students aged 11 to 16. It provides academic challenge and develops life skills during a critical period of young people's development. The MYP aims to motivate students, help them build on their strengths, embrace challenges, explore learning preferences, take appropriate risks, and develop a strong sense of personal identity. It is inclusive and designed as a whole-school activity preparing students for further study. The programme emphasizes holistic learning, intercultural awareness, communication, and international-mindedness aligned with the IB mission. It encourages personal, social, and emotional well-being alongside academic success, supporting students to become active, compassionate, and lifelong learners who appreciate diverse perspectives 12.
+1Approaches to learning and approaches to teaching in the Middle Years Programme_approaches-to-learning-and-approaches-to-teaching-in-the-mid-en_af9646cb-da0c-4a76-bc1d-4c127a5b7744.xml_12MYP: From principles into practice (Updated 2022 for use with the latest Programme standards and practices)_m_0_mypxx_guu_1405_10_e.pdf_6</v>
+      </c>
+      <c r="F48" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G48" t="str">
+        <v>2026-09-29T05:21:02.124Z</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49">
+        <v>48</v>
+      </c>
+      <c r="B49" t="str">
+        <v>All</v>
+      </c>
+      <c r="C49" t="str">
+        <v>All</v>
+      </c>
+      <c r="D49" t="str">
+        <v>Cuántas asignaturas de nivel superior deben tomar los alumnos que aplican al Diploma?</v>
+      </c>
+      <c r="E49" t="str">
+        <v>I'm sorry, I'm unable to process this request.</v>
+      </c>
+      <c r="F49" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G49" t="str">
+        <v>2026-09-29T05:21:14.602Z</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50">
+        <v>49</v>
+      </c>
+      <c r="B50" t="str">
+        <v>All</v>
+      </c>
+      <c r="C50" t="str">
+        <v>All</v>
+      </c>
+      <c r="D50" t="str">
+        <v>How is the grade for TOK marked? Is TOK exhibition equivalent to an internal assessment?</v>
+      </c>
+      <c r="E50" t="str">
+        <v>I'm sorry, I'm unable to process this request.</v>
+      </c>
+      <c r="F50" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G50" t="str">
+        <v>2026-09-29T05:21:29.860Z</v>
+      </c>
+    </row>
+    <row r="51" xml:space="preserve">
+      <c r="A51">
+        <v>50</v>
+      </c>
+      <c r="B51" t="str">
+        <v>All</v>
+      </c>
+      <c r="C51" t="str">
+        <v>All</v>
+      </c>
+      <c r="D51" t="str">
+        <v>when should students write the tok essay?</v>
+      </c>
+      <c r="E51" t="str" xml:space="preserve">
+        <v xml:space="preserve">_x001b_[2mexpect(_x001b_[22m_x001b_[31mreceived_x001b_[39m_x001b_[2m)._x001b_[22mtoBeGreaterThan_x001b_[2m(_x001b_[22m_x001b_[32mexpected_x001b_[39m_x001b_[2m)_x001b_[22m
+Expected: &gt; _x001b_[32m47_x001b_[39m
+Received:   _x001b_[31m47_x001b_[39m
+Call Log:
+- Timeout 180000ms exceeded while waiting on the predicate</v>
+      </c>
+      <c r="F51" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="G51" t="str">
+        <v>2026-09-29T05:24:35.374Z</v>
+      </c>
+    </row>
+    <row r="52" xml:space="preserve">
+      <c r="A52">
+        <v>51</v>
+      </c>
+      <c r="B52" t="str">
+        <v>All</v>
+      </c>
+      <c r="C52" t="str">
+        <v>All</v>
+      </c>
+      <c r="D52" t="str">
+        <v>what is the requisite for language ab initio ?</v>
+      </c>
+      <c r="E52" t="str" xml:space="preserve">
+        <v xml:space="preserve">Language ab initio is designed for students with no prior experience or very limited previous exposure to the target language. It is important that students placed in language ab initio are genuine beginners; those who can already understand and respond to spoken and written language on a range of common topics should not be placed in this course, as it would not provide an appropriate academic challenge. Language ab initio is offered at Standard Level (SL) only 12.
+1Language ab initio guide (First assessment 2020)_d_2_anlan_gui_1802_3_e.pdf_82Language ab initio guide (First assessment 2020)_d_2_anlan_gui_1802_3_e.pdf_7</v>
+      </c>
+      <c r="F52" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G52" t="str">
+        <v>2026-09-29T05:24:50.021Z</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53">
+        <v>52</v>
+      </c>
+      <c r="B53" t="str">
+        <v>All</v>
+      </c>
+      <c r="C53" t="str">
+        <v>All</v>
+      </c>
+      <c r="D53" t="str">
+        <v>Es cierto que en el PYP el primer tema transdisciplinar debe ser siempre who we are_</v>
+      </c>
+      <c r="E53" t="str">
+        <v>I'm sorry, I'm unable to process this request.</v>
+      </c>
+      <c r="F53" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G53" t="str">
+        <v>2026-09-29T05:25:02.129Z</v>
+      </c>
+    </row>
+    <row r="54" xml:space="preserve">
+      <c r="A54">
+        <v>53</v>
+      </c>
+      <c r="B54" t="str">
+        <v>All</v>
+      </c>
+      <c r="C54" t="str">
+        <v>All</v>
+      </c>
+      <c r="D54" t="str">
+        <v>What are Programme Standards and Practices?</v>
+      </c>
+      <c r="E54" t="str" xml:space="preserve">
+        <v xml:space="preserve">Programme Standards and Practices are a foundational set of principles used by IB World Schools and the International Baccalaureate (IB) to ensure quality and fidelity in the implementation of IB programmes. They provide a set of criteria to evaluate the success of schools in implementing the four IB programmes: Primary Years Programme (PYP), Middle Years Programme (MYP), Diploma Programme (DP), and Career-related Programme (CP).
+These standards are general principles central to being an IB World School, while practices offer further definitions of the standards including guidance on their implementation. Requirements are more specific measures, including programme-specific elements called specifications, necessary for the successful delivery of each IB programme.
+The standards and practices are organized into four overarching categories: purpose, environment, culture, and learning. The framework places learning at the centre, surrounded by IB philosophy and the unique context of each school. This framework describes how the school community designs, develops, and evolves the programmes, emphasizing that all elements are interdependent and integrated within each school's unique context 12.
+1Programme standards and practices_2020-programme-standards-and-practices-en_271c712a-4a31-4b47-8020-f060c312cffc.xml_12Programme standards and practices (2014)_g_0_iboxx_amo_2208_1s_e.pdf_3</v>
+      </c>
+      <c r="F54" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G54" t="str">
+        <v>2026-09-29T05:25:20.445Z</v>
+      </c>
+    </row>
+    <row r="55" xml:space="preserve">
+      <c r="A55">
+        <v>54</v>
+      </c>
+      <c r="B55" t="str">
+        <v>All</v>
+      </c>
+      <c r="C55" t="str">
+        <v>All</v>
+      </c>
+      <c r="D55" t="str">
+        <v>What is a "requirement" in the PSP? Can you provide an example of one?</v>
+      </c>
+      <c r="E55" t="str" xml:space="preserve">
+        <v xml:space="preserve">In the Programme Standards and Practices (PSP), a "requirement" is a specific measure that schools must meet to successfully deliver an IB programme. Requirements are more detailed and concrete compared to standards and practices, often including programme-specific elements known as specifications.
+An example of a requirement is from the Diploma Programme (DP): the school must provide security for the storage, transportation, and/or transmission of IB assessment materials, whether physical or virtual, with controlled access restricted to designated staff. This ensures the integrity and confidentiality of assessment materials (DP 1) 1.
+1How to organize the self-study_d_0_iboxx_inf_2402_1ss_e.pdf_4</v>
+      </c>
+      <c r="F55" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G55" t="str">
+        <v>2026-09-29T05:25:32.378Z</v>
+      </c>
+    </row>
+    <row r="56" xml:space="preserve">
+      <c r="A56">
+        <v>55</v>
+      </c>
+      <c r="B56" t="str">
+        <v>All</v>
+      </c>
+      <c r="C56" t="str">
+        <v>All</v>
+      </c>
+      <c r="D56" t="str">
+        <v>can you provide a definition for PSP?</v>
+      </c>
+      <c r="E56" t="str" xml:space="preserve">
+        <v xml:space="preserve">Programme Standards and Practices (PSP) are a foundational set of principles used by IB World Schools and the International Baccalaureate (IB) to ensure quality and fidelity in the implementation of IB programmes. They provide criteria to evaluate the success of schools in implementing the four IB programmes: Primary Years Programme (PYP), Middle Years Programme (MYP), Diploma Programme (DP), and Career-related Programme (CP). PSP includes general standards that are central to being an IB World School, practices that further define these standards with guidance on implementation, and specific programme requirements necessary for successful delivery. The PSP framework is organized into four categories—purpose, environment, culture, and learning—with learning at the center, surrounded by IB philosophy and each school’s unique context, describing how the school community designs, develops, and evolves the programmes 1234.
+1Programme standards and practices_2020-programme-standards-and-practices-en_271c712a-4a31-4b47-8020-f060c312cffc.xml_12Understanding policy to practice in IB programmes_understanding-policy-to-practice-in-ib-programmes-en_117be521-e287-4edb-824e-8f78c48f7fca.xml_23How to organize the self-study_d_0_iboxx_inf_2402_1ss_e.pdf_174Programme standards and practices (2014)_g_0_iboxx_amo_2208_1s_e.pdf_3</v>
+      </c>
+      <c r="F56" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G56" t="str">
+        <v>2026-09-29T05:25:44.754Z</v>
+      </c>
+    </row>
+    <row r="57" xml:space="preserve">
+      <c r="A57">
+        <v>56</v>
+      </c>
+      <c r="B57" t="str">
+        <v>All</v>
+      </c>
+      <c r="C57" t="str">
+        <v>All</v>
+      </c>
+      <c r="D57" t="str">
+        <v>Is there an IB mission document?</v>
+      </c>
+      <c r="E57" t="str" xml:space="preserve">
+        <v xml:space="preserve">Yes, there is an IB mission document. The International Baccalaureate (IB) mission statement aims to develop inquiring, knowledgeable, and caring young people who help create a better and more peaceful world through intercultural understanding and respect. This mission is central to all IB programmes and shapes their educational philosophy and objectives 123.
+1What is an IB education?_what-is-an-ib-education-en_148279a4-dd5d-4552-bd1c-187c8442d91c.xml_12What is an IB education? support material_what-is-an-ib-education-support-material-en_8e64a303-5f54-4de8-861e-4e6afb31c104.xml_13What is an IB education?_what-is-an-ib-education-fr_b0eef3cc-0d10-41d0-85c4-f6dc1a7affbb.xml_1</v>
+      </c>
+      <c r="F57" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G57" t="str">
+        <v>2026-09-29T05:25:57.011Z</v>
+      </c>
+    </row>
+    <row r="58" xml:space="preserve">
+      <c r="A58">
+        <v>57</v>
+      </c>
+      <c r="B58" t="str">
+        <v>All</v>
+      </c>
+      <c r="C58" t="str">
+        <v>All</v>
+      </c>
+      <c r="D58" t="str">
+        <v>According tothe IB, can formative assessments be graded?</v>
+      </c>
+      <c r="E58" t="str" xml:space="preserve">
+        <v xml:space="preserve">According to the IB, formative assessments are primarily intended to provide detailed feedback to help develop students' capabilities rather than to assign grades. While formative assessment focuses on identifying students' strengths and weaknesses to support learning, it is generally not aimed at producing numeric marks or grades. Instead, formative assessments emphasize feedback that is actionable, timely, and personalized to promote student agency and improve learning. Grading is more associated with summative assessment, which measures what a candidate can do, often to demonstrate completion or readiness to progress. Therefore, formative assessments can include descriptive comments and feedback rather than formal grades, although they may sometimes be marked descriptively rather than numerically to support learning 12.
+1Assessment principles and practices—Quality assessments in a digital age_assessment-principles-and-practices-quality-assessments-in-a-en_17c00909-8e8a-4c7c-a8e4-f0e00e8004e6.xml_112Assessment principles and practices—Quality assessments in a digital age_assessment-principles-and-practices-quality-assessments-in-a-en_17c00909-8e8a-4c7c-a8e4-f0e00e8004e6.xml_35</v>
+      </c>
+      <c r="F58" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G58" t="str">
+        <v>2026-09-29T05:26:09.507Z</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59">
+        <v>58</v>
+      </c>
+      <c r="B59" t="str">
+        <v>All</v>
+      </c>
+      <c r="C59" t="str">
+        <v>All</v>
+      </c>
+      <c r="D59" t="str">
+        <v>Is there a limit to the number of meetings between personal project students and their supervisors?</v>
+      </c>
+      <c r="E59" t="str">
+        <v>I'm sorry, I'm unable to process this request.</v>
+      </c>
+      <c r="F59" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G59" t="str">
+        <v>2026-09-29T05:26:21.710Z</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60">
+        <v>59</v>
+      </c>
+      <c r="B60" t="str">
+        <v>All</v>
+      </c>
+      <c r="C60" t="str">
+        <v>All</v>
+      </c>
+      <c r="D60" t="str">
+        <v>Tell me the difference between a Internal Assessment SL and HL in maths AA</v>
+      </c>
+      <c r="E60" t="str">
+        <v>I'm sorry, I'm unable to process this request.</v>
+      </c>
+      <c r="F60" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G60" t="str">
+        <v>2026-09-29T05:26:37.062Z</v>
+      </c>
+    </row>
+    <row r="61" xml:space="preserve">
+      <c r="A61">
+        <v>60</v>
+      </c>
+      <c r="B61" t="str">
+        <v>All</v>
+      </c>
+      <c r="C61" t="str">
+        <v>All</v>
+      </c>
+      <c r="D61" t="str">
+        <v>can you summarize the key elements a school's Academic Integrity policy ought to include?</v>
+      </c>
+      <c r="E61" t="str" xml:space="preserve">
+        <v xml:space="preserve">A school's Academic Integrity policy should include the following key elements:
+Clear expectations and responsibilities: It should define academic integrity as a guiding principle, emphasizing honesty, trust, fairness, respect, and responsibility for all members of the school community 123.
+Embedding academic integrity into school culture: The policy must be integrated into the school’s structure and strategy, fostering an ethical culture rather than just listing rules or penalties 14.
+Communication and accessibility: The policy should be clearly communicated, accessible, and understandable to students, teachers, leadership, and parents/legal guardians, with age-appropriate language reflecting learners' developmental needs 24.
+Support for teaching and learning: It should include provisions to teach students the skills of citing and referencing, ethical use of information and tools (including AI), and produce authentic work 24.
+Procedures for misconduct and maladministration: The policy must outline what constitutes academic misconduct and school maladministration, and describe fair and consistent procedures to address transgressions 14.
+Ongoing review and development: Schools should regularly review and update the policy collaboratively to ensure it remains effective and aligned with IB expectations 4.
+Building understanding and awareness: The policy should promote understanding of academic integrity’s purpose, encouraging responsible behavior rather than relying solely on detection or punishment 15.
+1Academic integrity policy_academic-integrity-policy-en_d1fbfeab-1d1e-4349-96aa-a314410bc760.xml_42Academic integrity policy_academic-integrity-policy-en_d1fbfeab-1d1e-4349-96aa-a314410bc760.xml_243Academic integrity policy_academic-integrity-policy-en_d1fbfeab-1d1e-4349-96aa-a314410bc760.xml_14Academic integrity policy_academic-integrity-policy-en_d1fbfeab-1d1e-4349-96aa-a314410bc760.xml_235Academic integrity policy_academic-integrity-policy-en_d1fbfeab-1d1e-4349-96aa-a314410bc760.xml_22</v>
+      </c>
+      <c r="F61" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G61" t="str">
+        <v>2026-09-29T05:26:52.655Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G61"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added questions sheet client
</commit_message>
<xml_diff>
--- a/results/chatbot-results.xlsx
+++ b/results/chatbot-results.xlsx
@@ -422,7 +422,7 @@
         <v>timestamp</v>
       </c>
     </row>
-    <row r="2" xml:space="preserve">
+    <row r="2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -435,18 +435,17 @@
       <c r="D2" t="str">
         <v>What is the MYP? *</v>
       </c>
-      <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">The Middle Years Programme (MYP) is a comprehensive curriculum framework developed by the International Baccalaureate (IB) for students aged 11 to 16. It provides academic challenge and supports the development of life skills during a critical period of young people's growth, helping them build personal strengths, embrace challenges, and develop a strong sense of personal identity. The MYP emphasizes holistic learning, intercultural awareness, communication, and prepares students for further successful study. It is inclusive, designed to benefit all students, and organized around eight subject groups with a concept-driven and inquiry-based curriculum. The programme also includes important projects like the community project and personal project that develop students' skills in service and reflection, preparing them for future education and life experiences 123.
-1MYP: From principles into practice (Updated 2022 for use with the latest Programme standards and practices)_m_0_mypxx_guu_1405_10_e.pdf_62MYP: From principles into practice 2014 (For candidate schools following the 2014 Programme standards and practices authorization process)_m_0_mypxx_guu_2209_1_e.pdf_83Community project guide_myp-community-project-guide-en_1ab030ac-869b-4052-b2bd-f1bfe6aa2240.xml_2</v>
+      <c r="E2" t="str">
+        <v/>
       </c>
       <c r="F2" t="str">
         <v>PASS</v>
       </c>
       <c r="G2" t="str">
-        <v>2026-09-29T05:02:57.547Z</v>
-      </c>
-    </row>
-    <row r="3" xml:space="preserve">
+        <v>2026-09-29T07:15:48.022Z</v>
+      </c>
+    </row>
+    <row r="3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -459,18 +458,17 @@
       <c r="D3" t="str">
         <v>i need the descriptors ST</v>
       </c>
-      <c r="E3" t="str" xml:space="preserve">
-        <v xml:space="preserve">Subject-specific grade descriptors in the MYP serve as important references in the assessment process. They describe student performance at each grade level for each MYP subject group, aligning with criterion-related assessment philosophy. Teachers use these descriptors to predict student outcomes in eAssessment, ensuring alignment between teacher expectations and IB assessment results. The grade award team uses these descriptors to set grade boundaries, comparing student performance against descriptors at key grade transitions (e.g., grades 2 to 3, 3 to 4, and 6 to 7). This process helps standardize assessment across subjects and sessions by referencing real student work 1.
-1Interdisciplinary teaching and learning in the MYP (for use from September 2021/January 2022)_interdisciplinary-teaching-and-learning-in-the-myp-guide-en_1700f2b5-ce51-4dae-b272-c75303fca437.xml_24</v>
+      <c r="E3" t="str">
+        <v>Could you please clarify what you mean by "descriptors ST"? Are you referring to subject-specific grade descriptors or another type of descriptors within the IB Middle Years Programme? This will help me provide the most relevant information for you.</v>
       </c>
       <c r="F3" t="str">
         <v>PASS</v>
       </c>
       <c r="G3" t="str">
-        <v>2026-09-29T05:03:09.315Z</v>
-      </c>
-    </row>
-    <row r="4" xml:space="preserve">
+        <v>2026-09-29T07:15:59.293Z</v>
+      </c>
+    </row>
+    <row r="4">
       <c r="A4">
         <v>3</v>
       </c>
@@ -483,18 +481,17 @@
       <c r="D4" t="str">
         <v>Is there anything specific for PYP? AF</v>
       </c>
-      <c r="E4" t="str" xml:space="preserve">
-        <v xml:space="preserve">Yes, the Primary Years Programme (PYP) is specifically designed for students aged 3 to 12 and focuses on the development of the whole child as an inquirer both inside and outside the classroom. It is a curriculum framework guided by six transdisciplinary themes of global significance, explored through six subject areas and approaches to learning with a strong emphasis on inquiry. The PYP supports early learning through a constructivist and social constructivist approach, encouraging active exploration and play to foster cognitive and social-emotional development. It also values early learning as a crucial stage in brain development and lifelong learning foundation. The PYP is flexible to accommodate local curriculum demands and emphasizes international-mindedness, action, and inquiry-based learning tailored to young learners' developmental needs 123.
-1PYP principles for learning and teaching (video transcript, June 2016)_p_0_pypxx_crr_1606_1_e.pdf_12The early years in the PYP_the-early-years-in-the-pyp-en_9ea4bfa4-cb65-4dae-833c-57f40d6d93b7.xml_13IB and the ELA Common Core State Standards—Relationship studies: Resources to inform curriculum alignment_g_0_iboxx_amo_1308_1e_e.pdf_4</v>
+      <c r="E4" t="str">
+        <v>locator.count: Target page, context or browser has been closed</v>
       </c>
       <c r="F4" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G4" t="str">
-        <v>2026-09-29T05:03:20.557Z</v>
-      </c>
-    </row>
-    <row r="5" xml:space="preserve">
+        <v>2026-09-29T07:16:13.502Z</v>
+      </c>
+    </row>
+    <row r="5">
       <c r="A5">
         <v>4</v>
       </c>
@@ -507,18 +504,17 @@
       <c r="D5" t="str">
         <v>I want documents that support conceptual understanding ST</v>
       </c>
-      <c r="E5" t="str" xml:space="preserve">
-        <v xml:space="preserve">Conceptual understanding in IB programmes, including the MYP and PYP, is a central educational goal focusing on transforming personal understanding and collaborative meaning-making rather than rote memorization. Concepts are defined as "big ideas" that are enduring and transcend specific subjects or times, enabling students to explore significant issues and ideas. They promote deeper understanding, interdisciplinary connections, and critical and creative thinking skills. In the MYP, conceptual understanding involves key and related concepts that provide both breadth and depth, helping students co-construct meaning and develop transferability of knowledge and responsibility for their learning. Teaching through concepts encourages a broad, inclusive approach to education across national and cultural boundaries, supporting interdisciplinary learning and engagement with complex ideas 1.
-1MYP: From principles into practice 2014 (For candidate schools following the 2014 Programme standards and practices authorization process)_m_0_mypxx_guu_2209_1_e.pdf_16</v>
+      <c r="E5" t="str">
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F5" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G5" t="str">
-        <v>2026-09-29T05:03:31.777Z</v>
-      </c>
-    </row>
-    <row r="6" xml:space="preserve">
+        <v>2026-09-29T07:16:13.511Z</v>
+      </c>
+    </row>
+    <row r="6">
       <c r="A6">
         <v>5</v>
       </c>
@@ -531,21 +527,17 @@
       <c r="D6" t="str">
         <v>scope and sequence \ST</v>
       </c>
-      <c r="E6" t="str" xml:space="preserve">
-        <v xml:space="preserve">_x001b_[2mexpect(_x001b_[22m_x001b_[31mreceived_x001b_[39m_x001b_[2m)._x001b_[22mtoBeGreaterThan_x001b_[2m(_x001b_[22m_x001b_[32mexpected_x001b_[39m_x001b_[2m)_x001b_[22m
-Expected: &gt; _x001b_[32m4_x001b_[39m
-Received:   _x001b_[31m4_x001b_[39m
-Call Log:
-- Timeout 180000ms exceeded while waiting on the predicate</v>
+      <c r="E6" t="str">
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F6" t="str">
         <v>FAIL</v>
       </c>
       <c r="G6" t="str">
-        <v>2026-09-29T05:06:32.204Z</v>
-      </c>
-    </row>
-    <row r="7" xml:space="preserve">
+        <v>2026-09-29T07:16:13.521Z</v>
+      </c>
+    </row>
+    <row r="7">
       <c r="A7">
         <v>6</v>
       </c>
@@ -558,18 +550,17 @@
       <c r="D7" t="str">
         <v>learning progressions ST</v>
       </c>
-      <c r="E7" t="str" xml:space="preserve">
-        <v xml:space="preserve">Learning progressions in the IB context describe the development of skills, understanding, and capabilities as students increase their proficiency in a particular area. They serve as tools to help teachers identify students' current learning stages, recognize gaps, and plan the next achievable steps to advance learning. These progressions integrate cognitive and measurement sciences, linking curriculum, assessment, and instruction to provide coherence and support student growth. They emphasize starting from the learner's existing understanding, actively involving learners, developing metacognition, and recognizing the social aspects of learning. Learning progressions align with the IB’s emphasis on student agency and support a social constructivist approach, making learning visible and actionable for both educators and learners. Specifically, in the Primary Years Programme (PYP), learning progressions offer a framework for describing skills that represent an IB learner within subjects, supporting schools in designing customized scope and sequence documents that reflect their contexts. These progressions also act as bridges between curriculum, assessment, and pedagogy, enabling coherent and developmentally appropriate learning experiences across age groups 12345.
-1Learning progressions: Research report (April 2021)_p_0_pypxx_sur-ir_2104_1l_e.pdf_12Learning progressions: Research report (April 2021)_p_0_pypxx_sur-ir_2104_1l_e.pdf_53Learning progressions: Research report (April 2021)_p_0_pypxx_sur-ir_2104_1l_e.pdf_24Inquiry learning progressions: Introduction_inquiry-learning-progressions-introduction-en_63f5ac5f-ebbf-43e2-9d91-2ae3d88c6ca8.xml_15Learning progressions: Research report (April 2021)_p_0_pypxx_sur-ir_2104_1l_e.pdf_4</v>
+      <c r="E7" t="str">
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F7" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G7" t="str">
-        <v>2026-09-29T05:06:43.516Z</v>
-      </c>
-    </row>
-    <row r="8" xml:space="preserve">
+        <v>2026-09-29T07:16:13.529Z</v>
+      </c>
+    </row>
+    <row r="8">
       <c r="A8">
         <v>7</v>
       </c>
@@ -582,18 +573,17 @@
       <c r="D8" t="str">
         <v>I there any seperate document or a page in PYP which talks about approaches to teaching ST</v>
       </c>
-      <c r="E8" t="str" xml:space="preserve">
-        <v xml:space="preserve">Yes, there is a specific focus on "approaches to teaching" within the Primary Years Programme (PYP). It is described as part of the curriculum cycle — written, taught, and assessed — and emphasizes authentic learning that is inquiry-based and conceptually driven. This is discussed in the context of PYP's review themes, highlighting how learning is most effective when connected to the real world around students rather than contrived school tasks 1. Additionally, the PYP: From principles into practice document elaborates on the organizing structure of the programme, including learning and teaching approaches that support learner agency and inquiry-based education 2.
-1Consultation paper: An invitation to PYP Heads, coordinators and educators at IB World Schools to comment on key themes for the PYP review process. (January 2014)_p_0_pypxx_crr_1402_1_e.pdf_12Transition guide for the Primary Years Programme_p_0_pypxx_mph_1806_1_e.pdf_2</v>
+      <c r="E8" t="str">
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F8" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G8" t="str">
-        <v>2026-09-29T05:06:55.319Z</v>
-      </c>
-    </row>
-    <row r="9" xml:space="preserve">
+        <v>2026-09-29T07:16:13.536Z</v>
+      </c>
+    </row>
+    <row r="9">
       <c r="A9">
         <v>8</v>
       </c>
@@ -606,18 +596,17 @@
       <c r="D9" t="str">
         <v>Pyp exhibition AF</v>
       </c>
-      <c r="E9" t="str" xml:space="preserve">
-        <v xml:space="preserve">The PYP exhibition is a significant culminating learning experience in the Primary Years Programme where students demonstrate their understanding through an in-depth inquiry into issues or opportunities they have chosen to explore. It involves students taking responsibility for their learning by planning, sharing, and assessing their work collaboratively with peers and mentors. The exhibition showcases student agency and community engagement, emphasizing international-mindedness and action. It may be integrated as one of the six units of inquiry in the final year or conducted as a separate inquiry project, with flexibility for schools to adapt it to their context. Students initiate, design, and collaborate throughout the exhibition process, developing knowledge, skills, and conceptual understanding. Assessment focuses on reflection and documentation rather than grading, and schools are encouraged to move from guided to student-led exhibitions over several years to support growing student independence 1234.
-1PYP: From principles into practice FAQs_p_0_pypxx_faq_2008_4_e.pdf_52The learner_the-learner-en_a698410d-e95a-452f-bc70-ecc544da2ae4.xml_163PYP: From principles into practice FAQs_p_0_pypxx_faq_2008_4_e.pdf_64The Learner in the enhanced PYP_p_0_pypxx_amo_1711_1_e.pdf_5</v>
+      <c r="E9" t="str">
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F9" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G9" t="str">
-        <v>2026-09-29T05:07:10.546Z</v>
-      </c>
-    </row>
-    <row r="10" xml:space="preserve">
+        <v>2026-09-29T07:16:13.543Z</v>
+      </c>
+    </row>
+    <row r="10">
       <c r="A10">
         <v>9</v>
       </c>
@@ -630,21 +619,14 @@
       <c r="D10" t="str">
         <v>what are the 5 ATL ? ST</v>
       </c>
-      <c r="E10" t="str" xml:space="preserve">
-        <v xml:space="preserve">The five Approaches to Learning (ATL) skill categories identified in IB programmes are:
-Communication
-Social
-Self-management
-Research
-Thinking
-These categories encompass various skill clusters that help students learn how to learn, develop independence, collaborate, and reflect effectively 123.
-1Approaches to teaching and learning in the Diploma Programme_approaches-to-teaching-and-learning-in-the-diploma-programme-en_72487a02-2ee8-4cac-a7f2-3519bcd20703.xml_32Approaches to learning and approaches to teaching in the Middle Years Programme_approaches-to-learning-and-approaches-to-teaching-in-the-mid-en_af9646cb-da0c-4a76-bc1d-4c127a5b7744.xml_33MYP: From principles into practice (Updated 2022 for use with the latest Programme standards and practices)_m_0_mypxx_guu_1405_10_e.pdf_21</v>
+      <c r="E10" t="str">
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F10" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G10" t="str">
-        <v>2026-09-29T05:07:22.097Z</v>
+        <v>2026-09-29T07:16:13.548Z</v>
       </c>
     </row>
     <row r="11">
@@ -661,16 +643,16 @@
         <v>stand alone subjects PYP  AF</v>
       </c>
       <c r="E11" t="str">
-        <v/>
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F11" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G11" t="str">
-        <v>2026-09-29T05:08:04.527Z</v>
-      </c>
-    </row>
-    <row r="12" xml:space="preserve">
+        <v>2026-09-29T07:16:13.557Z</v>
+      </c>
+    </row>
+    <row r="12">
       <c r="A12">
         <v>11</v>
       </c>
@@ -683,26 +665,17 @@
       <c r="D12" t="str">
         <v>How can schools ensure academic honesty and ethical use of AI tools such as ChatGPT in DP and MYP assessments?</v>
       </c>
-      <c r="E12" t="str" xml:space="preserve">
-        <v xml:space="preserve">Schools can ensure academic honesty and the ethical use of AI tools like ChatGPT in DP and MYP assessments by implementing several key strategies:
-Develop and enforce an academic honesty policy aligned with IB expectations, tailored to the school's context and priorities, which clearly addresses the use of AI tools 1.
-Provide detailed guidance and staff development on academic writing, referencing systems, plagiarism, and the ethical use of AI tools to clarify expectations for both teachers and students 12.
-Require students to acknowledge AI-generated content by including in-text citations and bibliographic references specifying the AI tool used, the prompt given, and the date of generation, ensuring transparency and proper attribution 23.
-Engage students in discussions about academic integrity as an ethical choice, including the responsible use of emerging technologies, privacy, bias, and accountability, to foster critical thinking and ethical awareness 24.
-Use assessment design strategies such as selecting unique, specific, or localized topics that encourage original inquiry and reduce opportunities for plagiarism or reliance on ready-made AI outputs 1.
-Monitor and support students' use of AI tools, encouraging prompt history documentation to verify authenticity and improve students' skills in using AI responsibly 2.
-Ensure school policies on AI use are clear, communicated, and consistently applied, while teachers exercise professional judgment on the appropriate use of AI in learning and assessment contexts 524.
-Together, these approaches help maintain academic integrity while embracing the educational potential of AI technologies in IB programmes.
-1IB position paper: Academic honesty in the IB_g_0_ibres_sur-dr_1209_1a_e.pdf_62Reflective project teacher support material (first teaching 2025)_cp-reflective-project-tsm-2025-en_ac05169d-d5c9-4f6c-989f-c42854416389.xml_123Key points to explain the use of Artificial Intelligence (AI) tools (one page fact sheet)_g_0_malpr_sup_2305_2_e.pdf_14Academic integrity policy_academic-integrity-policy-en_d1fbfeab-1d1e-4349-96aa-a314410bc760.xml_255Personal and professional skills teacher support material (first teaching 2025)_cp-personal-and-professional-skills-tsm-2025-en_f0592814-2fb3-4c52-a9a5-fc63dd1ff082.xml_8</v>
+      <c r="E12" t="str">
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F12" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G12" t="str">
-        <v>2026-09-29T05:08:18.817Z</v>
-      </c>
-    </row>
-    <row r="13" xml:space="preserve">
+        <v>2026-09-29T07:16:13.563Z</v>
+      </c>
+    </row>
+    <row r="13">
       <c r="A13">
         <v>12</v>
       </c>
@@ -715,18 +688,17 @@
       <c r="D13" t="str">
         <v>will we still have related concepts</v>
       </c>
-      <c r="E13" t="str" xml:space="preserve">
-        <v xml:space="preserve">Yes, related concepts continue to be an important part of the IB curriculum framework. In the Primary Years Programme (PYP), students encounter key and related concepts, and in the Middle Years Programme (MYP) and Diploma Programme (DP), students further develop these conceptual understandings. Related concepts support inquiry into significant ideas and help students make connections across subjects and contexts, contributing to a deeper and more connected learning experience 1.
-1MYP: From principles into practice (Updated 2022 for use with the latest Programme standards and practices)_m_0_mypxx_guu_1405_10_e.pdf_15</v>
+      <c r="E13" t="str">
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F13" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G13" t="str">
-        <v>2026-09-29T05:08:30.512Z</v>
-      </c>
-    </row>
-    <row r="14" xml:space="preserve">
+        <v>2026-09-29T07:16:13.570Z</v>
+      </c>
+    </row>
+    <row r="14">
       <c r="A14">
         <v>13</v>
       </c>
@@ -739,25 +711,17 @@
       <c r="D14" t="str">
         <v>How can an IB World School effectively implement and evaluate ATL skills, student agency, inquiry-based learning, inclusion, academic integrity, multilingualism, and ethical AI use across the PYP, MYP, and DP while ensuring alignment with IB standards, collaborative planning, assessment practices, and evaluation visit expectations?</v>
       </c>
-      <c r="E14" t="str" xml:space="preserve">
-        <v xml:space="preserve">To effectively implement and evaluate Approaches to Learning (ATL) skills, student agency, inquiry-based learning, inclusion, academic integrity, multilingualism, and ethical AI use across PYP, MYP, and DP, an IB World School should adopt a comprehensive, collaborative, and reflective approach aligned with IB standards:
-Collaborative Planning and Integration: Schools should create time and structures for teachers to collaborate horizontally and vertically, ensuring ATL skills and other key elements are embedded consistently across subjects and year levels. This involves shared planning meetings, interdisciplinary units, and coordinated curriculum maps reflecting ATL progression and inquiry-based learning approaches 1.
-Community Involvement and Partnerships: Engaging counselors, librarians, parents, and coordinators as allies in supporting ATL development, study skills, academic honesty, and ethical practices is essential. Counselors can coach students on balance and stress management, while librarians support information literacy, academic honesty, and research skills. Parents can reinforce reflective practices and ethical use of technology at home 23.
-Clear Policies and Guidance: Developing and communicating detailed academic honesty policies aligned with IB expectations ensures learners understand integrity requirements, including managing plagiarism and appropriate use of AI tools. Providing students with guidelines on citations and ethical AI use fosters transparency and responsibility 4.
-Formative and Summative Assessment Practices: Implement assessment strategies that promote student agency and self-assessment, encouraging learners to reflect on their ATL skill development and inquiry processes. Use assessment for learning principles to adapt teaching responsively and provide meaningful feedback, supporting inclusive learning environments 53.
-Monitoring and Reflection: Regular self-assessment and reflection by students on their ATL skills and learning progress enhance motivation and ownership. Schools can include these reflections in reporting and use them to inform curriculum adjustments and professional development 3.
-Alignment with IB Standards and Evaluation: Documenting collaborative planning, ATL skill integration, academic honesty practices, and inclusive strategies provides evidence for IB programme standards and evaluation visits. Maintaining clear records of planning agendas, unit plans, policy documents, and examples of student work supports the evaluation process 14.
-By embedding these elements systematically and fostering a school-wide culture of ethical, inquiry-driven, and inclusive learning, IB World Schools can uphold IB principles and meet programme expectations effectively.
-1Further guidance for developing ATL in the MYP_m_0_mypxx_fcl_1409_1a_e.pdf_42Approaches to teaching and learning in the Diploma Programme_approaches-to-teaching-and-learning-in-the-diploma-programme-en_72487a02-2ee8-4cac-a7f2-3519bcd20703.xml_313Approaches to teaching and learning in the Diploma Programme_approaches-to-teaching-and-learning-in-the-diploma-programme-en_72487a02-2ee8-4cac-a7f2-3519bcd20703.xml_304IB position paper: Academic honesty in the IB_g_0_ibres_sur-dr_1209_1a_e.pdf_15Teaching and learning informed by assessment in the Diploma Programme_teaching-and-learning-informed-by-assessment-in-the-diploma--en_a8ba94f8-e0ea-4c2c-b2d7-c578850fec35.xml_1</v>
+      <c r="E14" t="str">
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F14" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G14" t="str">
-        <v>2026-09-29T05:08:51.822Z</v>
-      </c>
-    </row>
-    <row r="15" xml:space="preserve">
+        <v>2026-09-29T07:16:13.583Z</v>
+      </c>
+    </row>
+    <row r="15">
       <c r="A15">
         <v>14</v>
       </c>
@@ -770,19 +734,17 @@
       <c r="D15" t="str">
         <v>am I allowed to use the term "IB Prep" or "pre-IB" for classes in a junior program leading the DP, and we have MYP.</v>
       </c>
-      <c r="E15" t="str" xml:space="preserve">
-        <v xml:space="preserve">The retrieved IB documentation does not provide specific guidelines regarding the use of terms like "IB Prep" or "pre-IB" for classes in a junior program leading to the Diploma Programme (DP), especially when the school already offers the Middle Years Programme (MYP). Generally, schools authorized to offer IB programmes follow IB terminology and frameworks to maintain clarity and alignment with IB standards.
-To ensure compliance and avoid confusion, it is recommended that schools consult directly with their IB regional office or IB coordinator for guidance on appropriate naming conventions for programs preparing students for the DP, particularly when the MYP is already offered as the official junior programme 12.
-1Middle Years Programme Assessment procedures 2025_myp-assessment-procedures-2025-en_5b9e6038-e524-4797-9e5e-57b70799783e.xml_72Middle Years Programme Assessment procedures 2026_myp-assessment-procedures-2026-en_ec81f7c7-2942-4e7c-ac96-a18447c2ca3e.xml_7</v>
+      <c r="E15" t="str">
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F15" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G15" t="str">
-        <v>2026-09-29T05:09:06.681Z</v>
-      </c>
-    </row>
-    <row r="16" xml:space="preserve">
+        <v>2026-09-29T07:16:13.587Z</v>
+      </c>
+    </row>
+    <row r="16">
       <c r="A16">
         <v>15</v>
       </c>
@@ -795,22 +757,14 @@
       <c r="D16" t="str">
         <v>give me details on implementing an MYP interdisciplinary unit</v>
       </c>
-      <c r="E16" t="str" xml:space="preserve">
-        <v xml:space="preserve">Implementing an MYP interdisciplinary unit involves several key steps to ensure meaningful integration of disciplines and rigorous student learning:
-Purpose and Inquiry: Begin by establishing a clear, meaningful purpose for the interdisciplinary unit that aligns with the MYP philosophy and requirements. This includes identifying a real-world issue or challenge that benefits from integrating multiple disciplines. Teachers collaboratively decide on the driving questions and the product or outcome students will create, ensuring the integration is purposeful and not superficial 12.
-Planning: Use the MYP interdisciplinary unit planner, a stand-alone document designed to organize interdisciplinary teaching and learning. The planner supports teamwork and collaboration among teachers from different disciplines. Teachers select key and related concepts, global contexts, and inquiry questions (factual, conceptual, and debatable) that frame the unit 13.
-Collaboration and Reflection: Teachers work collaboratively to develop the unit plan, discussing probing questions to deepen understanding of the interdisciplinary learning process. Reviewing example unit plans at different development levels can help refine the quality of planning over time 24.
-Assessment: Develop assessment tasks using MYP interdisciplinary criteria, focusing on integration of disciplines and ATL skills. Employ diverse strategies such as observations, student journals, and portfolio analysis to collect evidence of student learning. Collaboration among teachers in assessment is important to leverage disciplinary expertise 2.
-Implementation: Deliver the unit with an emphasis on inquiry-based, concept-driven learning, ensuring students understand the purpose of integration and how different disciplines contribute to addressing the real-world issue 52.
-Support and Resources: Teachers are encouraged to use IB eAssessment materials and teacher support materials (TSM) as practical guides for planning and teaching interdisciplinary units 24.
-Following these steps helps schools create interdisciplinary units that are meaningful, rigorous, and aligned with the MYP framework, fostering students' ability to integrate knowledge and skills across disciplines 51324.
-1Interdisciplinary teaching and learning in the MYP (for use from September 2021/January 2022)_interdisciplinary-teaching-and-learning-in-the-myp-guide-en_1700f2b5-ce51-4dae-b272-c75303fca437.xml_122Interdisciplinary teaching and learning in the MYP (for use from September 2021/January 2022)_interdisciplinary-teaching-and-learning-in-the-myp-guide-en_1700f2b5-ce51-4dae-b272-c75303fca437.xml_203Interdisciplinary teaching and learning in the MYP (for use from September 2021/January 2022)_interdisciplinary-teaching-and-learning-in-the-myp-guide-en_1700f2b5-ce51-4dae-b272-c75303fca437.xml_114Interdisciplinary teaching and learning in the MYP teacher support material_interdisciplinary-teaching-and-learning-in-the-myp-tsm-en_8037eec6-6d4a-465c-aed4-04ebe1484ed2.xml_15Interdisciplinary teaching and learning in the MYP (for use from September 2021/January 2022)_interdisciplinary-teaching-and-learning-in-the-myp-guide-en_1700f2b5-ce51-4dae-b272-c75303fca437.xml_1</v>
+      <c r="E16" t="str">
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F16" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G16" t="str">
-        <v>2026-09-29T05:09:27.706Z</v>
+        <v>2026-09-29T07:16:13.594Z</v>
       </c>
     </row>
     <row r="17">
@@ -827,13 +781,13 @@
         <v>when is MYP resources expected to be available on IB Exchange?</v>
       </c>
       <c r="E17" t="str">
-        <v>The retrieved documents do not provide specific information regarding the expected availability date of MYP resources on IB Exchange. For the most accurate and up-to-date details, it is recommended to consult the IB Programme Resource Centre or contact your IB regional office directly.</v>
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F17" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G17" t="str">
-        <v>2026-09-29T05:09:43.059Z</v>
+        <v>2026-09-29T07:16:13.598Z</v>
       </c>
     </row>
     <row r="18">
@@ -850,16 +804,16 @@
         <v>Why can't you process these requests? What did I do wrong?</v>
       </c>
       <c r="E18" t="str">
-        <v>You haven't done anything wrong. The information you provided relates mostly to AI and its impact on learning, inquiry, and knowledge, but it doesn't include details about the IB's policies or procedures regarding processing requests or submissions. Therefore, I don't have the necessary IB-specific context to answer questions about why certain IB requests might not be processed. For questions about IB administrative processes or technical issues, please contact your IB coordinator or the official IB support channels for assistance.</v>
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F18" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G18" t="str">
-        <v>2026-09-29T05:09:54.640Z</v>
-      </c>
-    </row>
-    <row r="19" xml:space="preserve">
+        <v>2026-09-29T07:16:13.604Z</v>
+      </c>
+    </row>
+    <row r="19">
       <c r="A19">
         <v>18</v>
       </c>
@@ -872,18 +826,17 @@
       <c r="D19" t="str">
         <v>Where can I get sample papers for MYP1 to MYP4?</v>
       </c>
-      <c r="E19" t="str" xml:space="preserve">
-        <v xml:space="preserve">Sample papers for MYP mathematics and other subjects for MYP1 to MYP4 can be accessed through the IB's Programme Resource Centre (PRC) available on My IB. Specifically, you can find teaching materials and teacher support materials which include examples and sample questions to guide your planning. For mathematics, the teacher support material provides examples applying MYP mathematics suggested by schools worldwide, which can be helpful for preparing assessment tasks for various criteria 1.
-1Mathematics: Frequently asked questions from the webinar “How to help your students thrive during the MYP mathematics eAssessment”_m_5_mathm_faq_2403_1_e.pdf_7</v>
+      <c r="E19" t="str">
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F19" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G19" t="str">
-        <v>2026-09-29T05:10:06.659Z</v>
-      </c>
-    </row>
-    <row r="20" xml:space="preserve">
+        <v>2026-09-29T07:16:13.611Z</v>
+      </c>
+    </row>
+    <row r="20">
       <c r="A20">
         <v>19</v>
       </c>
@@ -896,21 +849,17 @@
       <c r="D20" t="str">
         <v>WOuld you like to tell me more about MYP language and literature key topics/themes that are covered in MYP 4?</v>
       </c>
-      <c r="E20" t="str" xml:space="preserve">
-        <v xml:space="preserve">In MYP Language and Literature, including MYP 4, the curriculum emphasizes developing students' appreciation and understanding of language and literature through key concepts such as communication, connections, creativity, and perspective. These concepts are explored in greater depth as students progress, with related discipline-specific concepts introduced to suit their academic development stage.
-The course encourages the development of six interrelated skill areas: listening, speaking, reading, writing, viewing, and presenting. It promotes analytical and organizational skills in creative, personal, and imaginative ways, fostering intercultural understanding and engagement at local, national, and global levels.
-While there are no prescribed texts, teachers select a broad range of literary and non-literary texts that suit students' interests and needs, broaden their experiences, enhance historical and intercultural understanding, and model effective communication across diverse audiences and purposes. The curriculum is flexible and culturally sensitive, supporting international-mindedness.
-These elements prepare students for the Diploma Programme studies in language and literature, ensuring a smooth transition and continued development of linguistic and literary skills 12345.
-1Language A: language and literature guide_language-a-language-and-literature-guide-first-assessment-20-en_45a3922b-b147-478c-9f00-78cbf1fea859.xml_102Language A: literature guide_language-a-literature-guide-first-assessment-2021-en_f1795501-4f95-400c-960c-6c4b91a12e25.xml_103Language A: language and literature guide_language-a-language-and-literature-guide-first-assessment-20-en_45a3922b-b147-478c-9f00-78cbf1fea859.xml_114Language A: literature guide_language-a-literature-guide-first-assessment-2021-en_f1795501-4f95-400c-960c-6c4b91a12e25.xml_115Language and literature guide (for use from September 2014/January 2015)_m_1_langa_guu_1405_8_e.pdf_36</v>
+      <c r="E20" t="str">
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F20" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G20" t="str">
-        <v>2026-09-29T05:10:24.964Z</v>
-      </c>
-    </row>
-    <row r="21" xml:space="preserve">
+        <v>2026-09-29T07:16:13.615Z</v>
+      </c>
+    </row>
+    <row r="21">
       <c r="A21">
         <v>20</v>
       </c>
@@ -923,22 +872,14 @@
       <c r="D21" t="str">
         <v>math summative assessment</v>
       </c>
-      <c r="E21" t="str" xml:space="preserve">
-        <v xml:space="preserve">In the MYP, mathematics summative assessments are designed to evaluate student achievement based on specific subject-group assessment criteria, which include:
-Criterion A: Knowing and understanding
-Criterion B: Investigating patterns
-Criterion C: Communicating
-Criterion D: Applying mathematics in real-life contexts
-Each criterion is scored with a maximum of 8 marks, and assessments are structured to allow students to demonstrate their skills and understanding across these areas 1.
-Summative assessments are integral to the learning process and should be aligned with subject-group objectives, providing authentic opportunities for students to show their knowledge and skills. They can be designed as a single task assessing multiple criteria or multiple related tasks assessing different criteria, with increasing complexity as students progress through the MYP years 23.
-For external verification, MYP students may take optional on-screen examinations (eAssessment), which follow an examination blueprint ensuring consistency and alignment with the assessment criteria. These eAssessments simulate classroom internal assessments and provide a balanced measure of student achievement 1.
-1Mathematics guide (for use from September 2020/January 2021)_mathematics-guide-for-use-from-september-2020january-2021-en_f972b695-a0a4-43b9-a744-dfce17c03b9f.xml_152MYP: From principles into practice (Updated 2022 for use with the latest Programme standards and practices)_m_0_mypxx_guu_1405_10_e.pdf_713Further guidance for developing MYP assessed curriculum_m_0_mypxx_fcl_1409_3b_e.pdf_3</v>
+      <c r="E21" t="str">
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F21" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G21" t="str">
-        <v>2026-09-29T05:10:39.460Z</v>
+        <v>2026-09-29T07:16:13.620Z</v>
       </c>
     </row>
     <row r="22" xml:space="preserve">
@@ -963,16 +904,16 @@
 Naoki Kobayashi</v>
       </c>
       <c r="E22" t="str">
-        <v/>
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F22" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G22" t="str">
-        <v>2026-09-29T05:11:28.140Z</v>
-      </c>
-    </row>
-    <row r="23" xml:space="preserve">
+        <v>2026-09-29T07:16:13.625Z</v>
+      </c>
+    </row>
+    <row r="23">
       <c r="A23">
         <v>22</v>
       </c>
@@ -985,19 +926,17 @@
       <c r="D23" t="str">
         <v>called to ask if they can have an IB elective class added to their curriculum. The class would not count towards the 8 disciplines for the MYP, and would not fall under any specific subject. I advised I will escalate to curriculum.</v>
       </c>
-      <c r="E23" t="str" xml:space="preserve">
-        <v xml:space="preserve">In the MYP, students are generally expected to study courses from at least six subject groups concurrently in years 4 and 5, including language and literature, language acquisition, individuals and societies, sciences, mathematics, and one additional subject group (arts, design, or physical and health education) 1. While schools have flexibility to combine subject groups or offer electives, any additional courses outside the core subject groups typically do not count towards the required eight disciplines for the MYP certificate 12.
-Offering an IB elective class that does not fall under a specific subject group and does not contribute to the core MYP subject requirements is possible, but it would be considered outside the formal MYP subject-group framework. Such an elective would be an addition to the curriculum rather than part of the assessed MYP disciplines. It is appropriate to escalate this request to curriculum coordinators to ensure alignment with IB programme requirements and school policies 12.
-1MYP: From principles into practice 2014 (For candidate schools following the 2014 Programme standards and practices authorization process)_m_0_mypxx_guu_2209_1_e.pdf_422Interdisciplinary teaching and learning in the MYP (for use from September 2021/January 2022)_interdisciplinary-teaching-and-learning-in-the-myp-guide-en_1700f2b5-ce51-4dae-b272-c75303fca437.xml_3</v>
+      <c r="E23" t="str">
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F23" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G23" t="str">
-        <v>2026-09-29T05:11:42.621Z</v>
-      </c>
-    </row>
-    <row r="24" xml:space="preserve">
+        <v>2026-09-29T07:16:13.633Z</v>
+      </c>
+    </row>
+    <row r="24">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1010,18 +949,17 @@
       <c r="D24" t="str">
         <v>ATL framework</v>
       </c>
-      <c r="E24" t="str" xml:space="preserve">
-        <v xml:space="preserve">The Approaches to Learning (ATL) framework in the MYP is a central element designed to develop students' learning skills across all subjects and years. It consists of five broad categories of ATL skills that support students in becoming effective, independent learners. These skills are both subject-specific and general, inclusive of "soft skills," and aligned with the IB learner profile values. Schools are expected to plan for the vertical (across years) and horizontal (across subjects) articulation of ATL skills to ensure meaningful progression and coordination of students' learning experiences. The framework is intended to be integral to unit planning and owned by students to promote lifelong learning abilities. While schools are not required to report on all ATL skills formally, meaningful feedback and self-evaluation of ATL skill development are encouraged to enhance student growth. Collaborative planning among teachers and structured time for horizontal planning are important to support the effective implementation of ATL skills in the curriculum. The ATL planning can be organized flexibly, using charts or other documents, and may be informed by external standards or frameworks to scaffold skill development progressively throughout the MYP 12345.
-1Further guidance for developing ATL in the MYP_m_0_mypxx_fcl_1409_1a_e.pdf_12Further guidance for developing ATL in the MYP_m_0_mypxx_fcl_1409_1a_e.pdf_33Further guidance for developing ATL in the MYP_m_0_mypxx_fcl_1409_1a_e.pdf_44Further guidance for developing ATL in the MYP_m_0_mypxx_fcl_1409_1a_e.pdf_85Further guidance for developing ATL in the MYP_m_0_mypxx_fcl_1409_1a_e.pdf_6</v>
+      <c r="E24" t="str">
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F24" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G24" t="str">
-        <v>2026-09-29T05:11:57.813Z</v>
-      </c>
-    </row>
-    <row r="25" xml:space="preserve">
+        <v>2026-09-29T07:16:13.644Z</v>
+      </c>
+    </row>
+    <row r="25">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1034,21 +972,17 @@
       <c r="D25" t="str">
         <v>Can you a frame a question where all 4 programms are interrelated? frame any 2</v>
       </c>
-      <c r="E25" t="str" xml:space="preserve">
-        <v xml:space="preserve">Here are two example questions that interrelate all four IB programmes (PYP, MYP, DP, and CP) by focusing on connected, interdisciplinary learning and global contexts:
-How can the concept of sustainability be explored and addressed across different disciplines and IB programmes, from early inquiry in the PYP through interdisciplinary projects in the MYP, to advanced research in the DP and career-related applications in the CP?
-In what ways can international-mindedness and global citizenship be developed through the transdisciplinary themes of the PYP, conceptual and connected curriculum in the MYP, theory of knowledge and extended essay investigations in the DP, and reflective projects in the CP?
-These questions emphasize the continuum of learning across programmes, highlighting the increasing disciplinary complexity and integration while maintaining a connected and holistic educational experience 1234.
-1Interdisciplinary teaching and learning in the MYP (for use from September 2021/January 2022)_interdisciplinary-teaching-and-learning-in-the-myp-guide-en_1700f2b5-ce51-4dae-b272-c75303fca437.xml_32Interdisciplinary teaching and learning in the MYP (for use from September 2021/January 2022)_interdisciplinary-teaching-and-learning-in-the-myp-guide-en_1700f2b5-ce51-4dae-b272-c75303fca437.xml_43Interdisciplinary teaching and learning in the MYP (for use from September 2021/January 2022)_interdisciplinary-teaching-and-learning-in-the-myp-guide-en_1700f2b5-ce51-4dae-b272-c75303fca437.xml_54What is an IB education?_what-is-an-ib-education-en_148279a4-dd5d-4552-bd1c-187c8442d91c.xml_3</v>
+      <c r="E25" t="str">
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F25" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G25" t="str">
-        <v>2026-09-29T05:12:13.228Z</v>
-      </c>
-    </row>
-    <row r="26" xml:space="preserve">
+        <v>2026-09-29T07:16:13.650Z</v>
+      </c>
+    </row>
+    <row r="26">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1061,24 +995,17 @@
       <c r="D26" t="str">
         <v>what are the requirements to receive your CP certificate</v>
       </c>
-      <c r="E26" t="str" xml:space="preserve">
-        <v xml:space="preserve">To receive the IB Career-related Programme (CP) certificate, a student must satisfactorily complete several requirements including:
-Completion of the specified career-related study.
-Achieving a grade of 3 or higher in at least two Diploma Programme (DP) courses.
-Earning a grade of D or higher on the reflective project.
-Meeting the requirements for personal and professional skills, service learning (minimum 50 hours), and language development (minimum 50 hours).
-Not receiving any penalties for academic misconduct.
-Upon meeting these conditions, students are awarded the IB CP Certificate along with a statement of results detailing their achievements in DP courses, the reflective project, and the status of CP core completion 123.
-1Career-related Programme Assessment procedures 2026_cp-assessment-procedures-2026-en_bd9462b2-fc3e-40db-be74-b80152ab95e2.xml_52Letter to accompany university application Career-related Programme, 2025_d_x_carec_grad_2409_2_e.pdf_23Career-related Programme Assessment procedures 2026_cp-assessment-procedures-2026-en_bd9462b2-fc3e-40db-be74-b80152ab95e2.xml_10</v>
+      <c r="E26" t="str">
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F26" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G26" t="str">
-        <v>2026-09-29T05:12:28.272Z</v>
-      </c>
-    </row>
-    <row r="27" xml:space="preserve">
+        <v>2026-09-29T07:16:13.655Z</v>
+      </c>
+    </row>
+    <row r="27">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1091,18 +1018,17 @@
       <c r="D27" t="str">
         <v>what does sustained engagement over the duration of the Cp mean in practical terms</v>
       </c>
-      <c r="E27" t="str" xml:space="preserve">
-        <v xml:space="preserve">In practical terms, "sustained engagement over the duration of the CP" means that students consistently participate and remain actively involved in all components of the Career-related Programme throughout the entire period of study (typically ages 16 to 19). This includes continuous commitment to their career-related study, Diploma Programme courses, the CP core components (such as the reflective project, language development, service learning, and personal and professional skills), and related assessments. Sustained engagement requires students to demonstrate ongoing effort, time management, and development of skills and knowledge rather than sporadic or minimal involvement, ensuring they meet the learning outcomes and requirements of the CP framework 12.
-1Community engagement guide (first teaching 2025)_cp-community-engagement-guide-2025-en_91e189b0-9664-4328-b3eb-dfe61b281fb9.xml_12Career-related Programme Assessment procedures 2026_cp-assessment-procedures-2026-en_bd9462b2-fc3e-40db-be74-b80152ab95e2.xml_2</v>
+      <c r="E27" t="str">
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F27" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G27" t="str">
-        <v>2026-09-29T05:12:43.020Z</v>
-      </c>
-    </row>
-    <row r="28" xml:space="preserve">
+        <v>2026-09-29T07:16:13.658Z</v>
+      </c>
+    </row>
+    <row r="28">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1115,21 +1041,17 @@
       <c r="D28" t="str">
         <v>What are the differences between IBDP and IBCP?</v>
       </c>
-      <c r="E28" t="str" xml:space="preserve">
-        <v xml:space="preserve">The International Baccalaureate Diploma Programme (IBDP) and the Career-related Programme (IBCP) differ primarily in focus and structure:
-IBDP is a two-year academic programme for students aged 16-19 that offers a broad and challenging curriculum across six subject groups. It emphasizes interdisciplinary understanding, critical thinking, and preparation for university-level study. Students take courses at standard or higher level, complete core components like the Extended Essay and Theory of Knowledge, and aim for the full IB Diploma 12.
-IBCP is designed for students aged 16-19 who want to combine academic study with career-related learning. It includes at least two Diploma Programme courses, a career-related study (which is not offered or awarded by the IB but must meet IB criteria), and a distinctive CP core that develops personal and professional skills, service learning, language development, and a reflective project. The CP prepares students for higher education, apprenticeships, or employment by integrating applied knowledge and practical skills with academic rigor 324.
-In summary, the IBDP is more academic and broad-based, while the IBCP offers a flexible framework combining academic courses with career-related education and skills development.
-1Research report— Postsecondary outcomes of International Baccalaureate Diploma Programme graduates in the United States (2024)_g_0_ibres_sur-ir_2406_1a_e.pdf_22Research report— Postsecondary outcomes of International Baccalaureate Career-related Programme graduates in the United States (2024)_g_0_ibres_sur-ir_2406_1_e.pdf_23Letter to accompany university application Career-related Programme, 2025_d_x_carec_grad_2409_2_e.pdf_14Overview of the Career-related Programme_d_0_carec_amo-16_1512_1_e.pdf_3</v>
+      <c r="E28" t="str">
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F28" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G28" t="str">
-        <v>2026-09-29T05:12:57.746Z</v>
-      </c>
-    </row>
-    <row r="29" xml:space="preserve">
+        <v>2026-09-29T07:16:13.663Z</v>
+      </c>
+    </row>
+    <row r="29">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1142,18 +1064,17 @@
       <c r="D29" t="str">
         <v>what planner do i use for the PYP exhibition AF</v>
       </c>
-      <c r="E29" t="str" xml:space="preserve">
-        <v xml:space="preserve">For the PYP exhibition, you use the PYP planner as outlined in Making the PYP Happen: A Curriculum Framework for International Primary Education (2009). Each exhibition must be documented on a PYP planner if it is included within the programme of inquiry. However, schools have the flexibility to implement the exhibition outside of the programme of inquiry, in which case a PYP planner is not required. This flexibility allows schools to adapt the exhibition to their context while supporting student agency and inquiry 123.
-1Coordinator’s handbook 2013 - 2014_p_0_pypxx_coh_1308_1_e.pdf_392PYP: From principles into practice FAQs_p_0_pypxx_faq_2008_4_e.pdf_63The Learner in the enhanced PYP_p_0_pypxx_amo_1711_1_e.pdf_6</v>
+      <c r="E29" t="str">
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F29" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G29" t="str">
-        <v>2026-09-29T05:13:10.085Z</v>
-      </c>
-    </row>
-    <row r="30" xml:space="preserve">
+        <v>2026-09-29T07:16:13.673Z</v>
+      </c>
+    </row>
+    <row r="30">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1166,21 +1087,17 @@
       <c r="D30" t="str">
         <v>Nothing about age 3-6 learners? We have a lot of bilingual multilingual learners ST</v>
       </c>
-      <c r="E30" t="str" xml:space="preserve">
-        <v xml:space="preserve">_x001b_[2mexpect(_x001b_[22m_x001b_[31mreceived_x001b_[39m_x001b_[2m)._x001b_[22mtoBeGreaterThan_x001b_[2m(_x001b_[22m_x001b_[32mexpected_x001b_[39m_x001b_[2m)_x001b_[22m
-Expected: &gt; _x001b_[32m27_x001b_[39m
-Received:   _x001b_[31m27_x001b_[39m
-Call Log:
-- Timeout 180000ms exceeded while waiting on the predicate</v>
+      <c r="E30" t="str">
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F30" t="str">
         <v>FAIL</v>
       </c>
       <c r="G30" t="str">
-        <v>2026-09-29T05:16:14.087Z</v>
-      </c>
-    </row>
-    <row r="31" xml:space="preserve">
+        <v>2026-09-29T07:16:13.678Z</v>
+      </c>
+    </row>
+    <row r="31">
       <c r="A31">
         <v>30</v>
       </c>
@@ -1193,18 +1110,17 @@
       <c r="D31" t="str">
         <v>there are 3 strands in PSPE ST</v>
       </c>
-      <c r="E31" t="str" xml:space="preserve">
-        <v xml:space="preserve">Yes, the three strands in the PYP Personal, Social, and Physical Education (PSPE) are Identity, Active Living, and Interactions. These strands organize the learning continuums and provide a framework for developing conceptual understandings and learner outcomes across the phases of the programme 1.
-1PSPE development report: Second report for teachers (April 2022)_p_0_pypxx_sur_2204_3p_e.pdf_6</v>
+      <c r="E31" t="str">
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F31" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G31" t="str">
-        <v>2026-09-29T05:16:28.737Z</v>
-      </c>
-    </row>
-    <row r="32" xml:space="preserve">
+        <v>2026-09-29T07:16:13.684Z</v>
+      </c>
+    </row>
+    <row r="32">
       <c r="A32">
         <v>31</v>
       </c>
@@ -1217,20 +1133,17 @@
       <c r="D32" t="str">
         <v>are the approaches to teaching the same in the PYP and MYP ST</v>
       </c>
-      <c r="E32" t="str" xml:space="preserve">
-        <v xml:space="preserve">The approaches to teaching in the PYP and MYP share some underlying principles but are tailored to suit the developmental stages and specific aims of each programme. In the MYP, teaching styles are evolving from traditional subject-focused transmission to more skills-based, process-oriented methods that promote student self-regulation and engagement. This includes shared regulation between teacher and students and process-oriented instruction that supports independent learning and metacognitive skills development 12.
-In the PYP, teaching approaches emphasize transdisciplinary learning and designing curricula that integrate PSPE with other subjects, focusing on holistic development including play, relationships, and symbolic exploration in early years. The PYP also highlights the role of the teacher as a curriculum designer and uses IB approaches to teaching to support this design process 34.
-Therefore, while both programmes value student agency, inquiry, and skill development, the MYP has a stronger focus on transitioning students towards more andragogical, self-regulated learning styles as they mature, whereas the PYP emphasizes early holistic and transdisciplinary learning experiences 12.
-1Approaches to learning and approaches to teaching in the Middle Years Programme_approaches-to-learning-and-approaches-to-teaching-in-the-mid-en_af9646cb-da0c-4a76-bc1d-4c127a5b7744.xml_192Approaches to learning and approaches to teaching in the Middle Years Programme_approaches-to-learning-and-approaches-to-teaching-in-the-mid-en_af9646cb-da0c-4a76-bc1d-4c127a5b7744.xml_183PSPE development report: First report for teachers (April 2021)_p_0_pypxx_sur_2104_1p_e.pdf_54PSPE development report: First report for teachers (April 2021)_p_0_pypxx_sur_2104_1p_e.pdf_6</v>
+      <c r="E32" t="str">
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F32" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G32" t="str">
-        <v>2026-09-29T05:16:44.219Z</v>
-      </c>
-    </row>
-    <row r="33" xml:space="preserve">
+        <v>2026-09-29T07:16:13.688Z</v>
+      </c>
+    </row>
+    <row r="33">
       <c r="A33">
         <v>32</v>
       </c>
@@ -1243,18 +1156,17 @@
       <c r="D33" t="str">
         <v>can enviromental sciene be an interdisciplinary subject</v>
       </c>
-      <c r="E33" t="str" xml:space="preserve">
-        <v xml:space="preserve">Yes, Environmental Science can be an interdisciplinary subject. It combines methodologies and techniques from both experimental sciences and human sciences, reflecting its interdisciplinary nature. This allows students to explore ecological concepts, environmental laws, economics, and ethical considerations in a connected way. For example, students can study environmental issues using both qualitative and quantitative methods, investigate local or global problems, and apply knowledge from various disciplines to understand and address sustainability challenges 123.
-1Environmental systems and societies teacher support material_environmental-systems-teacher-support-material-en_c1c4de2e-8fe2-4f21-afb9-7531d9d1c45c.xml_32Environmental systems and societies teacher support material_environmental-systems-teacher-support-material-en_c1c4de2e-8fe2-4f21-afb9-7531d9d1c45c.xml_113Environmental systems and societies teacher support material_environmental-systems-teacher-support-material-en_c1c4de2e-8fe2-4f21-afb9-7531d9d1c45c.xml_23</v>
+      <c r="E33" t="str">
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F33" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G33" t="str">
-        <v>2026-09-29T05:16:58.912Z</v>
-      </c>
-    </row>
-    <row r="34" xml:space="preserve">
+        <v>2026-09-29T07:16:13.692Z</v>
+      </c>
+    </row>
+    <row r="34">
       <c r="A34">
         <v>33</v>
       </c>
@@ -1267,15 +1179,14 @@
       <c r="D34" t="str">
         <v>Are there any subject guides for the MYP beta</v>
       </c>
-      <c r="E34" t="str" xml:space="preserve">
-        <v xml:space="preserve">Yes, there are subject guides and enhanced curriculum content available as part of the Enhancing the MYP BETA trial. The trial provides updated curriculum guidance on unit planning and other components to support schools participating in the beta phase. Resources such as the Enhancing the MYP BETA trial website contain curriculum content and guidance, and workshops are offered to help educators engage with enhanced unit planning, curriculum design, and implementation strategies 12.
-1Enhancing the MYP: Making the MYP better for all students, teachers and school communities_enhancing-the-myp-making-the-myp-better-for-all-students-tea-en_a0dd97db-7c45-4106-a1bd-d6a515abcc9b.xml_22Middle Years Programme updates, May 2025_m_g_mypxx_con_2505_1_e.pdf_2</v>
+      <c r="E34" t="str">
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F34" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G34" t="str">
-        <v>2026-09-29T05:17:10.962Z</v>
+        <v>2026-09-29T07:16:13.697Z</v>
       </c>
     </row>
     <row r="35">
@@ -1292,13 +1203,13 @@
         <v>Is making mistakes in grammar in French B tested in criterion A ?</v>
       </c>
       <c r="E35" t="str">
-        <v>Yes, in French B, making mistakes in grammar is considered under Criterion A, which evaluates the student's linguistic competence. This includes vocabulary, grammatical structures, language accuracy, pronunciation, and intonation. Errors that interfere with communication, such as grammatical mistakes that make sentences incoherent or difficult to understand, affect the Criterion A assessment. However, minor errors that do not hinder understanding may have less impact on the mark .</v>
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F35" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G35" t="str">
-        <v>2026-09-29T05:17:32.418Z</v>
+        <v>2026-09-29T07:16:13.703Z</v>
       </c>
     </row>
     <row r="36">
@@ -1315,13 +1226,13 @@
         <v>is it mandatory to teach design?</v>
       </c>
       <c r="E36" t="str">
-        <v>I'm sorry, I'm unable to process this request.</v>
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F36" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G36" t="str">
-        <v>2026-09-29T05:17:44.479Z</v>
+        <v>2026-09-29T07:16:13.708Z</v>
       </c>
     </row>
     <row r="37">
@@ -1338,16 +1249,16 @@
         <v>do kids have to do teh eassessmsnt in myp 5</v>
       </c>
       <c r="E37" t="str">
-        <v>I'm sorry, I'm unable to process this request.</v>
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F37" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G37" t="str">
-        <v>2026-09-29T05:17:59.801Z</v>
-      </c>
-    </row>
-    <row r="38" xml:space="preserve">
+        <v>2026-09-29T07:16:13.713Z</v>
+      </c>
+    </row>
+    <row r="38">
       <c r="A38">
         <v>37</v>
       </c>
@@ -1360,18 +1271,17 @@
       <c r="D38" t="str">
         <v>can a student who has been in Lang Lit in MYP do Lang B in the same language in DP if they do not have the level for the Lang Lit in DP?</v>
       </c>
-      <c r="E38" t="str" xml:space="preserve">
-        <v xml:space="preserve">A student who has studied Language and Literature (Lang Lit) in the MYP but does not have the required level for Language and Literature in the Diploma Programme (DP) may consider taking Language B in the same language in the DP, provided their linguistic proficiency aligns better with Language B requirements. The MYP Language acquisition guide recommends that students achieve at least Phase 5 or Phase 6 in Language acquisition before progressing to DP studies in language and literature, and sometimes it is suggested that students have some MYP Language and Literature experience for a smoother transition. Ultimately, the choice between Language and Literature and Language B in the DP depends on the student’s language proficiency and should be made in consultation with teachers and coordinators to ensure an appropriate match to the student's skills and educational goals 12.
-1Language A: language and literature guide_d_1_alanl_gui_2507_1_e.pdf_162Language A: literature guide_d_1_alite_gui_2507_1_e.pdf_15</v>
+      <c r="E38" t="str">
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F38" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G38" t="str">
-        <v>2026-09-29T05:18:14.936Z</v>
-      </c>
-    </row>
-    <row r="39" xml:space="preserve">
+        <v>2026-09-29T07:16:13.719Z</v>
+      </c>
+    </row>
+    <row r="39">
       <c r="A39">
         <v>38</v>
       </c>
@@ -1384,18 +1294,17 @@
       <c r="D39" t="str">
         <v>When is the IBCP Refelctive Project turned into the IB?</v>
       </c>
-      <c r="E39" t="str" xml:space="preserve">
-        <v xml:space="preserve">The IB Career-related Programme (IBCP) Reflective Project is submitted towards the end of the Career-related Programme. Students work on it over an extended period, and it is expected that they devote a minimum of 50 hours to its completion. After the school assesses the Reflective Project, a sample is sent electronically to the IB for external moderation. The submission must be in one of the IB working languages (English, Spanish, or French), and live links are not permitted. The final submission includes the written essay (or essay plus an additional format) and the Reflections on Planning and Progress Form (RPPF) 123.
-1Reflective project guide (last assessment 2026)_d_0_carec_gui-16_1512_2r_e.pdf_102Reflective project teacher support material (last assessment 2026)_cp-reflective-project-tsm-2015-en_f954c3a4-289c-403e-8d7e-33f490aba326.xml_13Additional guidance for the reflective project (last assessment 2026)_d_0_carec_amo_1604_1_e.pdf_4</v>
+      <c r="E39" t="str">
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F39" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G39" t="str">
-        <v>2026-09-29T05:18:27.068Z</v>
-      </c>
-    </row>
-    <row r="40" xml:space="preserve">
+        <v>2026-09-29T07:16:13.723Z</v>
+      </c>
+    </row>
+    <row r="40">
       <c r="A40">
         <v>39</v>
       </c>
@@ -1408,18 +1317,17 @@
       <c r="D40" t="str">
         <v>hiw many hours are required</v>
       </c>
-      <c r="E40" t="str" xml:space="preserve">
-        <v xml:space="preserve">Students are expected to devote a minimum of 50 hours to complete the IB Career-related Programme Reflective Project over an extended period of time 123.
-1Reflective project guide (first teaching 2025)_cp-reflective-project-guide-2025-en_56cec644-bd5f-4ba1-a167-d7996151afc2.xml_72Reflective project guide (last assessment 2026)_d_0_carec_gui-16_1512_2r_e.pdf_73Reflective project guide (last assessment 2026)_d_0_carec_gui-16_1512_2r_e.pdf_6</v>
+      <c r="E40" t="str">
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F40" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G40" t="str">
-        <v>2026-09-29T05:18:39.389Z</v>
-      </c>
-    </row>
-    <row r="41" xml:space="preserve">
+        <v>2026-09-29T07:16:13.731Z</v>
+      </c>
+    </row>
+    <row r="41">
       <c r="A41">
         <v>40</v>
       </c>
@@ -1432,24 +1340,17 @@
       <c r="D41" t="str">
         <v>Tell me about assessing the IBCP core components</v>
       </c>
-      <c r="E41" t="str" xml:space="preserve">
-        <v xml:space="preserve">The assessment of the IB Career-related Programme (IBCP) core components involves evaluating the Reflective Project, which is externally assessed and focuses on an ethical dilemma related to the student's career-related studies. The assessment criteria include:
-Criterion A: Focus on the ethical dilemma — assessing how well the ethical dilemma is identified and explored from different perspectives and contexts.
-Criterion B: Knowledge and understanding through research — evaluating the use of research to develop understanding of the ethical dilemma and its impacts.
-Criterion C: Critical thinking — analyzing and synthesizing research to justify a personal position considering implications for various contexts and groups.
-Criterion D: Communication of ideas — assessing clarity, organization, terminology, and structure in communicating ideas.
-Criterion E: Reflective practice — evaluating the planning, research, and implementation of reflective practices during the project.
-The Reflective Project is externally moderated, and supervisors do not assign marks but may provide predicted grades based on qualitative grade descriptors. These descriptors guide understanding of the academic expectations and help in setting grade boundaries during moderation. Schools must also review and evaluate the delivery of all core components regularly to ensure relevance and integration, as part of ongoing quality assurance and programme evaluation processes 1.
-1Reflective project guide (first teaching 2025)_cp-reflective-project-guide-2025-en_56cec644-bd5f-4ba1-a167-d7996151afc2.xml_26</v>
+      <c r="E41" t="str">
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F41" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G41" t="str">
-        <v>2026-09-29T05:18:54.521Z</v>
-      </c>
-    </row>
-    <row r="42" xml:space="preserve">
+        <v>2026-09-29T07:16:13.742Z</v>
+      </c>
+    </row>
+    <row r="42">
       <c r="A42">
         <v>41</v>
       </c>
@@ -1462,18 +1363,17 @@
       <c r="D42" t="str">
         <v>is a language B required for the CP?</v>
       </c>
-      <c r="E42" t="str" xml:space="preserve">
-        <v xml:space="preserve">No, a Language B course is not specifically required for the IB Career-related Programme (CP). However, language development is a core component of the CP, ensuring that all students have access to and are exposed to an additional language. Students are encouraged to begin or extend the study of a language other than their best language to develop their linguistic and communicative abilities. A minimum of 50 hours is expected to be devoted to language development as part of the CP core, but this does not mandate a Language B course specifically 123.
-1Letter to accompany university application Career-related Programme, 2025_d_x_carec_grad_2409_2_e.pdf_22Career-related Programme Assessment procedures 2026_cp-assessment-procedures-2026-en_bd9462b2-fc3e-40db-be74-b80152ab95e2.xml_43Career-related Programme Assessment procedures 2026_cp-assessment-procedures-2026-en_bd9462b2-fc3e-40db-be74-b80152ab95e2.xml_5</v>
+      <c r="E42" t="str">
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F42" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G42" t="str">
-        <v>2026-09-29T05:19:06.351Z</v>
-      </c>
-    </row>
-    <row r="43" xml:space="preserve">
+        <v>2026-09-29T07:16:13.756Z</v>
+      </c>
+    </row>
+    <row r="43">
       <c r="A43">
         <v>42</v>
       </c>
@@ -1486,15 +1386,14 @@
       <c r="D43" t="str">
         <v>Community Engagement hours</v>
       </c>
-      <c r="E43" t="str" xml:space="preserve">
-        <v xml:space="preserve">Schools are expected to allocate a minimum of 30 guided hours for the Community Engagement (CE) component of the IB Career-related Programme (CP). These guided hours cover the introduction, orientation, ongoing guidance, and review points for CE. However, the total number of hours students actively engage with the community outside of guided learning is not specified, as the focus is on sustained and meaningful engagement rather than a set quantity of hours. Schools may provide additional hours beyond the minimum to support students’ aspirations for CE 1.
-1Community engagement guide (first teaching 2025)_cp-community-engagement-guide-2025-en_91e189b0-9664-4328-b3eb-dfe61b281fb9.xml_17</v>
+      <c r="E43" t="str">
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F43" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G43" t="str">
-        <v>2026-09-29T05:19:18.575Z</v>
+        <v>2026-09-29T07:16:13.773Z</v>
       </c>
     </row>
     <row r="44">
@@ -1511,16 +1410,16 @@
         <v>What kind of Language students can take in language devleopment in CP Programme</v>
       </c>
       <c r="E44" t="str">
-        <v>I'm sorry, I'm unable to process this request.</v>
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F44" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G44" t="str">
-        <v>2026-09-29T05:19:31.069Z</v>
-      </c>
-    </row>
-    <row r="45" xml:space="preserve">
+        <v>2026-09-29T07:16:13.779Z</v>
+      </c>
+    </row>
+    <row r="45">
       <c r="A45">
         <v>44</v>
       </c>
@@ -1533,15 +1432,14 @@
       <c r="D45" t="str">
         <v>Is there a guide for writing an assessment policy? ST</v>
       </c>
-      <c r="E45" t="str" xml:space="preserve">
-        <v xml:space="preserve">Yes, there is guidance for schools on developing an assessment policy. Constructing and implementing an assessment policy helps schools engage meaningfully with IB assessment expectations while considering their unique context. The process involves understanding IB principles, comparing them with the school's current practices, and synthesizing these into a policy document that reflects a common understanding within the school community. The policy should include a philosophy of assessment, detail assessment practices (both formative and summative), and explain how grading, recording, and reporting are handled. It should also address timelines, workloads, and communicate assessment purposes clearly to all stakeholders. The policy must be a living document, collaboratively written, and regularly reviewed to improve practice. Schools can find this guidance in IB resources such as "Guidelines for developing a school assessment policy in the Diploma Programme" and related programme guides 123.
-1Guidelines for developing a school assessment policy in the Diploma Programme_d_0_dpyyy_ass_1101_1_e.pdf_22MYP: From principles into practice (Updated 2022 for use with the latest Programme standards and practices)_m_0_mypxx_guu_1405_10_e.pdf_383Guidelines for developing a school assessment policy in the Diploma Programme_d_0_dpyyy_ass_1101_1_e.pdf_5</v>
+      <c r="E45" t="str">
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F45" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G45" t="str">
-        <v>2026-09-29T05:19:46.271Z</v>
+        <v>2026-09-29T07:16:13.786Z</v>
       </c>
     </row>
     <row r="46" xml:space="preserve">
@@ -1559,16 +1457,16 @@
 The IB learner profile represents a broad range of human capacities and responsibilities that encompass intellectual, personal, emotional, and social growth. It supports students in developing international-mindedness and taking action for positive change. Through inquiry and reflection, learners develop attributes such as being open-minded, caring, and principled, which are explored and revisited across the transdisciplinary themes and subject-spec</v>
       </c>
       <c r="E46" t="str">
-        <v/>
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F46" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G46" t="str">
-        <v>2026-09-29T05:20:32.156Z</v>
-      </c>
-    </row>
-    <row r="47" xml:space="preserve">
+        <v>2026-09-29T07:16:13.792Z</v>
+      </c>
+    </row>
+    <row r="47">
       <c r="A47">
         <v>46</v>
       </c>
@@ -1581,21 +1479,17 @@
       <c r="D47" t="str">
         <v>What is the difference between Maths AI and Maths AA?</v>
       </c>
-      <c r="E47" t="str" xml:space="preserve">
-        <v xml:space="preserve">The difference between Mathematics: Applications and Interpretation (AI) and Mathematics: Analysis and Approaches (AA) lies primarily in their focus and approach:
-Mathematics: Analysis and Approaches (AA) is designed for students who enjoy developing strong mathematical thinking and fluency in constructing mathematical arguments. It includes traditional pre-university topics such as functions, trigonometry, calculus, sequences and series, and proof by induction. AA emphasizes analytical expertise and mathematical problem solving, with a strong focus on justifying and communicating mathematical arguments. It also allows the use of technology but prioritizes understanding and constructing proofs. AA is suitable for students interested in STEM fields or who enjoy abstract and theoretical mathematics 12.
-Mathematics: Applications and Interpretation (AI) focuses on the practical application of mathematics to describe the world and solve real-life problems. It emphasizes mathematical modelling and the use of technology to explore and construct models. AI includes topics like calculus and statistics but is more oriented towards applied mathematics and data interpretation. This course suits students who prefer contextual and practical mathematics, often in data-rich environments 12.
-In summary, AA is more theoretical and proof-oriented, while AI is more applied and modelling-focused, catering to different student interests and future academic or career paths .
-1Mathematics: applications and interpretation guide_mathematics-applications-and-interpretation-guide-en_f67500d4-c8e4-4d84-b3b6-26ea0c58132b.xml_62Mathematics: analysis and approaches guide_mathematics-analysis-and-approaches-guide-en_6b6db2f8-f7ce-414b-a41a-c090a26d5888.xml_6</v>
+      <c r="E47" t="str">
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F47" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G47" t="str">
-        <v>2026-09-29T05:20:46.957Z</v>
-      </c>
-    </row>
-    <row r="48" xml:space="preserve">
+        <v>2026-09-29T07:16:13.797Z</v>
+      </c>
+    </row>
+    <row r="48">
       <c r="A48">
         <v>47</v>
       </c>
@@ -1608,15 +1502,14 @@
       <c r="D48" t="str">
         <v>What is the MYP?</v>
       </c>
-      <c r="E48" t="str" xml:space="preserve">
-        <v xml:space="preserve">The Middle Years Programme (MYP) is a comprehensive curriculum framework designed by the International Baccalaureate (IB) for students aged 11 to 16. It provides academic challenge and develops life skills during a critical period of young people's development. The MYP aims to motivate students, help them build on their strengths, embrace challenges, explore learning preferences, take appropriate risks, and develop a strong sense of personal identity. It is inclusive and designed as a whole-school activity preparing students for further study. The programme emphasizes holistic learning, intercultural awareness, communication, and international-mindedness aligned with the IB mission. It encourages personal, social, and emotional well-being alongside academic success, supporting students to become active, compassionate, and lifelong learners who appreciate diverse perspectives 12.
-1Approaches to learning and approaches to teaching in the Middle Years Programme_approaches-to-learning-and-approaches-to-teaching-in-the-mid-en_af9646cb-da0c-4a76-bc1d-4c127a5b7744.xml_12MYP: From principles into practice (Updated 2022 for use with the latest Programme standards and practices)_m_0_mypxx_guu_1405_10_e.pdf_6</v>
+      <c r="E48" t="str">
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F48" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G48" t="str">
-        <v>2026-09-29T05:21:02.124Z</v>
+        <v>2026-09-29T07:16:13.803Z</v>
       </c>
     </row>
     <row r="49">
@@ -1633,13 +1526,13 @@
         <v>Cuántas asignaturas de nivel superior deben tomar los alumnos que aplican al Diploma?</v>
       </c>
       <c r="E49" t="str">
-        <v>I'm sorry, I'm unable to process this request.</v>
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F49" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G49" t="str">
-        <v>2026-09-29T05:21:14.602Z</v>
+        <v>2026-09-29T07:16:13.808Z</v>
       </c>
     </row>
     <row r="50">
@@ -1656,16 +1549,16 @@
         <v>How is the grade for TOK marked? Is TOK exhibition equivalent to an internal assessment?</v>
       </c>
       <c r="E50" t="str">
-        <v>I'm sorry, I'm unable to process this request.</v>
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F50" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G50" t="str">
-        <v>2026-09-29T05:21:29.860Z</v>
-      </c>
-    </row>
-    <row r="51" xml:space="preserve">
+        <v>2026-09-29T07:16:13.814Z</v>
+      </c>
+    </row>
+    <row r="51">
       <c r="A51">
         <v>50</v>
       </c>
@@ -1678,21 +1571,17 @@
       <c r="D51" t="str">
         <v>when should students write the tok essay?</v>
       </c>
-      <c r="E51" t="str" xml:space="preserve">
-        <v xml:space="preserve">_x001b_[2mexpect(_x001b_[22m_x001b_[31mreceived_x001b_[39m_x001b_[2m)._x001b_[22mtoBeGreaterThan_x001b_[2m(_x001b_[22m_x001b_[32mexpected_x001b_[39m_x001b_[2m)_x001b_[22m
-Expected: &gt; _x001b_[32m47_x001b_[39m
-Received:   _x001b_[31m47_x001b_[39m
-Call Log:
-- Timeout 180000ms exceeded while waiting on the predicate</v>
+      <c r="E51" t="str">
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F51" t="str">
         <v>FAIL</v>
       </c>
       <c r="G51" t="str">
-        <v>2026-09-29T05:24:35.374Z</v>
-      </c>
-    </row>
-    <row r="52" xml:space="preserve">
+        <v>2026-09-29T07:16:13.819Z</v>
+      </c>
+    </row>
+    <row r="52">
       <c r="A52">
         <v>51</v>
       </c>
@@ -1705,15 +1594,14 @@
       <c r="D52" t="str">
         <v>what is the requisite for language ab initio ?</v>
       </c>
-      <c r="E52" t="str" xml:space="preserve">
-        <v xml:space="preserve">Language ab initio is designed for students with no prior experience or very limited previous exposure to the target language. It is important that students placed in language ab initio are genuine beginners; those who can already understand and respond to spoken and written language on a range of common topics should not be placed in this course, as it would not provide an appropriate academic challenge. Language ab initio is offered at Standard Level (SL) only 12.
-1Language ab initio guide (First assessment 2020)_d_2_anlan_gui_1802_3_e.pdf_82Language ab initio guide (First assessment 2020)_d_2_anlan_gui_1802_3_e.pdf_7</v>
+      <c r="E52" t="str">
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F52" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G52" t="str">
-        <v>2026-09-29T05:24:50.021Z</v>
+        <v>2026-09-29T07:16:13.823Z</v>
       </c>
     </row>
     <row r="53">
@@ -1730,16 +1618,16 @@
         <v>Es cierto que en el PYP el primer tema transdisciplinar debe ser siempre who we are_</v>
       </c>
       <c r="E53" t="str">
-        <v>I'm sorry, I'm unable to process this request.</v>
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F53" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G53" t="str">
-        <v>2026-09-29T05:25:02.129Z</v>
-      </c>
-    </row>
-    <row r="54" xml:space="preserve">
+        <v>2026-09-29T07:16:13.828Z</v>
+      </c>
+    </row>
+    <row r="54">
       <c r="A54">
         <v>53</v>
       </c>
@@ -1752,20 +1640,17 @@
       <c r="D54" t="str">
         <v>What are Programme Standards and Practices?</v>
       </c>
-      <c r="E54" t="str" xml:space="preserve">
-        <v xml:space="preserve">Programme Standards and Practices are a foundational set of principles used by IB World Schools and the International Baccalaureate (IB) to ensure quality and fidelity in the implementation of IB programmes. They provide a set of criteria to evaluate the success of schools in implementing the four IB programmes: Primary Years Programme (PYP), Middle Years Programme (MYP), Diploma Programme (DP), and Career-related Programme (CP).
-These standards are general principles central to being an IB World School, while practices offer further definitions of the standards including guidance on their implementation. Requirements are more specific measures, including programme-specific elements called specifications, necessary for the successful delivery of each IB programme.
-The standards and practices are organized into four overarching categories: purpose, environment, culture, and learning. The framework places learning at the centre, surrounded by IB philosophy and the unique context of each school. This framework describes how the school community designs, develops, and evolves the programmes, emphasizing that all elements are interdependent and integrated within each school's unique context 12.
-1Programme standards and practices_2020-programme-standards-and-practices-en_271c712a-4a31-4b47-8020-f060c312cffc.xml_12Programme standards and practices (2014)_g_0_iboxx_amo_2208_1s_e.pdf_3</v>
+      <c r="E54" t="str">
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F54" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G54" t="str">
-        <v>2026-09-29T05:25:20.445Z</v>
-      </c>
-    </row>
-    <row r="55" xml:space="preserve">
+        <v>2026-09-29T07:16:13.833Z</v>
+      </c>
+    </row>
+    <row r="55">
       <c r="A55">
         <v>54</v>
       </c>
@@ -1778,19 +1663,17 @@
       <c r="D55" t="str">
         <v>What is a "requirement" in the PSP? Can you provide an example of one?</v>
       </c>
-      <c r="E55" t="str" xml:space="preserve">
-        <v xml:space="preserve">In the Programme Standards and Practices (PSP), a "requirement" is a specific measure that schools must meet to successfully deliver an IB programme. Requirements are more detailed and concrete compared to standards and practices, often including programme-specific elements known as specifications.
-An example of a requirement is from the Diploma Programme (DP): the school must provide security for the storage, transportation, and/or transmission of IB assessment materials, whether physical or virtual, with controlled access restricted to designated staff. This ensures the integrity and confidentiality of assessment materials (DP 1) 1.
-1How to organize the self-study_d_0_iboxx_inf_2402_1ss_e.pdf_4</v>
+      <c r="E55" t="str">
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F55" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G55" t="str">
-        <v>2026-09-29T05:25:32.378Z</v>
-      </c>
-    </row>
-    <row r="56" xml:space="preserve">
+        <v>2026-09-29T07:16:13.839Z</v>
+      </c>
+    </row>
+    <row r="56">
       <c r="A56">
         <v>55</v>
       </c>
@@ -1803,18 +1686,17 @@
       <c r="D56" t="str">
         <v>can you provide a definition for PSP?</v>
       </c>
-      <c r="E56" t="str" xml:space="preserve">
-        <v xml:space="preserve">Programme Standards and Practices (PSP) are a foundational set of principles used by IB World Schools and the International Baccalaureate (IB) to ensure quality and fidelity in the implementation of IB programmes. They provide criteria to evaluate the success of schools in implementing the four IB programmes: Primary Years Programme (PYP), Middle Years Programme (MYP), Diploma Programme (DP), and Career-related Programme (CP). PSP includes general standards that are central to being an IB World School, practices that further define these standards with guidance on implementation, and specific programme requirements necessary for successful delivery. The PSP framework is organized into four categories—purpose, environment, culture, and learning—with learning at the center, surrounded by IB philosophy and each school’s unique context, describing how the school community designs, develops, and evolves the programmes 1234.
-1Programme standards and practices_2020-programme-standards-and-practices-en_271c712a-4a31-4b47-8020-f060c312cffc.xml_12Understanding policy to practice in IB programmes_understanding-policy-to-practice-in-ib-programmes-en_117be521-e287-4edb-824e-8f78c48f7fca.xml_23How to organize the self-study_d_0_iboxx_inf_2402_1ss_e.pdf_174Programme standards and practices (2014)_g_0_iboxx_amo_2208_1s_e.pdf_3</v>
+      <c r="E56" t="str">
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F56" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G56" t="str">
-        <v>2026-09-29T05:25:44.754Z</v>
-      </c>
-    </row>
-    <row r="57" xml:space="preserve">
+        <v>2026-09-29T07:16:13.844Z</v>
+      </c>
+    </row>
+    <row r="57">
       <c r="A57">
         <v>56</v>
       </c>
@@ -1827,18 +1709,17 @@
       <c r="D57" t="str">
         <v>Is there an IB mission document?</v>
       </c>
-      <c r="E57" t="str" xml:space="preserve">
-        <v xml:space="preserve">Yes, there is an IB mission document. The International Baccalaureate (IB) mission statement aims to develop inquiring, knowledgeable, and caring young people who help create a better and more peaceful world through intercultural understanding and respect. This mission is central to all IB programmes and shapes their educational philosophy and objectives 123.
-1What is an IB education?_what-is-an-ib-education-en_148279a4-dd5d-4552-bd1c-187c8442d91c.xml_12What is an IB education? support material_what-is-an-ib-education-support-material-en_8e64a303-5f54-4de8-861e-4e6afb31c104.xml_13What is an IB education?_what-is-an-ib-education-fr_b0eef3cc-0d10-41d0-85c4-f6dc1a7affbb.xml_1</v>
+      <c r="E57" t="str">
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F57" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G57" t="str">
-        <v>2026-09-29T05:25:57.011Z</v>
-      </c>
-    </row>
-    <row r="58" xml:space="preserve">
+        <v>2026-09-29T07:16:13.851Z</v>
+      </c>
+    </row>
+    <row r="58">
       <c r="A58">
         <v>57</v>
       </c>
@@ -1851,15 +1732,14 @@
       <c r="D58" t="str">
         <v>According tothe IB, can formative assessments be graded?</v>
       </c>
-      <c r="E58" t="str" xml:space="preserve">
-        <v xml:space="preserve">According to the IB, formative assessments are primarily intended to provide detailed feedback to help develop students' capabilities rather than to assign grades. While formative assessment focuses on identifying students' strengths and weaknesses to support learning, it is generally not aimed at producing numeric marks or grades. Instead, formative assessments emphasize feedback that is actionable, timely, and personalized to promote student agency and improve learning. Grading is more associated with summative assessment, which measures what a candidate can do, often to demonstrate completion or readiness to progress. Therefore, formative assessments can include descriptive comments and feedback rather than formal grades, although they may sometimes be marked descriptively rather than numerically to support learning 12.
-1Assessment principles and practices—Quality assessments in a digital age_assessment-principles-and-practices-quality-assessments-in-a-en_17c00909-8e8a-4c7c-a8e4-f0e00e8004e6.xml_112Assessment principles and practices—Quality assessments in a digital age_assessment-principles-and-practices-quality-assessments-in-a-en_17c00909-8e8a-4c7c-a8e4-f0e00e8004e6.xml_35</v>
+      <c r="E58" t="str">
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F58" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G58" t="str">
-        <v>2026-09-29T05:26:09.507Z</v>
+        <v>2026-09-29T07:16:13.857Z</v>
       </c>
     </row>
     <row r="59">
@@ -1876,13 +1756,13 @@
         <v>Is there a limit to the number of meetings between personal project students and their supervisors?</v>
       </c>
       <c r="E59" t="str">
-        <v>I'm sorry, I'm unable to process this request.</v>
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F59" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G59" t="str">
-        <v>2026-09-29T05:26:21.710Z</v>
+        <v>2026-09-29T07:16:13.861Z</v>
       </c>
     </row>
     <row r="60">
@@ -1899,16 +1779,16 @@
         <v>Tell me the difference between a Internal Assessment SL and HL in maths AA</v>
       </c>
       <c r="E60" t="str">
-        <v>I'm sorry, I'm unable to process this request.</v>
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F60" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G60" t="str">
-        <v>2026-09-29T05:26:37.062Z</v>
-      </c>
-    </row>
-    <row r="61" xml:space="preserve">
+        <v>2026-09-29T07:16:13.866Z</v>
+      </c>
+    </row>
+    <row r="61">
       <c r="A61">
         <v>60</v>
       </c>
@@ -1921,22 +1801,14 @@
       <c r="D61" t="str">
         <v>can you summarize the key elements a school's Academic Integrity policy ought to include?</v>
       </c>
-      <c r="E61" t="str" xml:space="preserve">
-        <v xml:space="preserve">A school's Academic Integrity policy should include the following key elements:
-Clear expectations and responsibilities: It should define academic integrity as a guiding principle, emphasizing honesty, trust, fairness, respect, and responsibility for all members of the school community 123.
-Embedding academic integrity into school culture: The policy must be integrated into the school’s structure and strategy, fostering an ethical culture rather than just listing rules or penalties 14.
-Communication and accessibility: The policy should be clearly communicated, accessible, and understandable to students, teachers, leadership, and parents/legal guardians, with age-appropriate language reflecting learners' developmental needs 24.
-Support for teaching and learning: It should include provisions to teach students the skills of citing and referencing, ethical use of information and tools (including AI), and produce authentic work 24.
-Procedures for misconduct and maladministration: The policy must outline what constitutes academic misconduct and school maladministration, and describe fair and consistent procedures to address transgressions 14.
-Ongoing review and development: Schools should regularly review and update the policy collaboratively to ensure it remains effective and aligned with IB expectations 4.
-Building understanding and awareness: The policy should promote understanding of academic integrity’s purpose, encouraging responsible behavior rather than relying solely on detection or punishment 15.
-1Academic integrity policy_academic-integrity-policy-en_d1fbfeab-1d1e-4349-96aa-a314410bc760.xml_42Academic integrity policy_academic-integrity-policy-en_d1fbfeab-1d1e-4349-96aa-a314410bc760.xml_243Academic integrity policy_academic-integrity-policy-en_d1fbfeab-1d1e-4349-96aa-a314410bc760.xml_14Academic integrity policy_academic-integrity-policy-en_d1fbfeab-1d1e-4349-96aa-a314410bc760.xml_235Academic integrity policy_academic-integrity-policy-en_d1fbfeab-1d1e-4349-96aa-a314410bc760.xml_22</v>
+      <c r="E61" t="str">
+        <v>locator.waitFor: Target page, context or browser has been closed</v>
       </c>
       <c r="F61" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G61" t="str">
-        <v>2026-09-29T05:26:52.655Z</v>
+        <v>2026-09-29T07:16:13.872Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>